<commit_message>
Updated test matrix to match current reality (#888)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1773323801" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1773323801" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1773323801" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1773323801"/>
+      <pm:revision xmlns:pm="smNativeData" day="1776900014" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1776900014" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1776900014" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1776900014"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="111">
   <si>
     <t>Context</t>
   </si>
@@ -115,10 +115,13 @@
     <t>As static variable</t>
   </si>
   <si>
+    <t>N</t>
+  </si>
+  <si>
     <t>Y</t>
   </si>
   <si>
-    <t>N</t>
+    <t>?</t>
   </si>
   <si>
     <t>As function parameters</t>
@@ -157,6 +160,9 @@
     <t>Constructor</t>
   </si>
   <si>
+    <t>leak</t>
+  </si>
+  <si>
     <t>Scenario</t>
   </si>
   <si>
@@ -283,7 +289,13 @@
     <t>Abort controller</t>
   </si>
   <si>
-    <t>Promise</t>
+    <t>Promise (int)</t>
+  </si>
+  <si>
+    <t>Promise (string)</t>
+  </si>
+  <si>
+    <t>Promise (plain object)</t>
   </si>
   <si>
     <t>Callback</t>
@@ -385,7 +397,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1773323801" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -400,7 +412,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1773323801" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -415,7 +427,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1773323801" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -431,7 +443,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1773323801" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -453,7 +465,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -464,7 +476,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -475,7 +487,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -486,7 +498,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -497,7 +509,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -508,7 +520,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -530,7 +542,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1773323801"/>
+          <pm:border xmlns:pm="smNativeData" id="1776900014"/>
         </ext>
       </extLst>
     </border>
@@ -549,7 +561,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1773323801">
+          <pm:border xmlns:pm="smNativeData" id="1776900014">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -571,7 +583,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1773323801">
+          <pm:border xmlns:pm="smNativeData" id="1776900014">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -595,7 +607,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1773323801">
+          <pm:border xmlns:pm="smNativeData" id="1776900014">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -619,7 +631,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1773323801">
+          <pm:border xmlns:pm="smNativeData" id="1776900014">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -643,7 +655,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1773323801"/>
+          <pm:border xmlns:pm="smNativeData" id="1776900014"/>
         </ext>
       </extLst>
     </border>
@@ -662,7 +674,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1773323801"/>
+          <pm:border xmlns:pm="smNativeData" id="1776900014"/>
         </ext>
       </extLst>
     </border>
@@ -675,7 +687,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -703,6 +715,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -712,13 +727,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="29">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -731,7 +746,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -742,7 +757,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -755,7 +770,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -766,7 +781,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -779,7 +794,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -790,7 +805,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -803,7 +818,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -814,7 +829,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -827,7 +842,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -838,7 +853,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -851,7 +866,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -862,7 +877,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -875,7 +890,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -886,7 +901,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -899,7 +914,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -910,7 +925,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -923,7 +938,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -934,7 +949,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -947,7 +962,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -958,7 +973,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -971,7 +986,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -982,7 +997,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -995,7 +1010,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1006,7 +1021,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1019,7 +1034,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1030,7 +1045,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1043,7 +1058,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1054,7 +1069,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1067,7 +1082,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1078,7 +1093,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1091,7 +1106,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1102,7 +1117,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1115,7 +1130,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1126,7 +1141,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1139,7 +1154,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1150,7 +1165,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1163,7 +1178,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1174,7 +1189,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1187,7 +1202,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1198,7 +1213,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1773323801" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1211,7 +1226,199 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1773323801" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1221,10 +1428,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1773323801" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1776900014" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1773323801" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1776900014" count="6">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -1493,7 +1700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:Y15"/>
+  <dimension ref="A1:Y17"/>
   <sheetFormatPr baseColWidth="7" defaultColWidth="8.544643" defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="22.151786" customWidth="1" style="0"/>
@@ -1637,19 +1844,19 @@
         <v>26</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>26</v>
@@ -1658,38 +1865,40 @@
         <v>26</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P3" s="10" t="s">
         <v>26</v>
       </c>
       <c r="Q3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S3" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T3" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T3" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V3" s="11"/>
       <c r="W3" s="11"/>
@@ -1697,187 +1906,191 @@
         <v>26</v>
       </c>
       <c r="Y3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="R4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="T4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="O4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="P4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="R4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="S4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T4" s="10"/>
       <c r="U4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V4" s="11"/>
       <c r="W4" s="11"/>
       <c r="X4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>26</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T5" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T5" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U5" s="10" t="s">
         <v>27</v>
       </c>
       <c r="V5" s="11"/>
       <c r="W5" s="11"/>
       <c r="X5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:25">
       <c r="A6" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I6" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M6" s="10" t="s">
         <v>26</v>
@@ -1886,10 +2099,10 @@
         <v>26</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q6" s="10" t="s">
         <v>26</v>
@@ -1898,11 +2111,13 @@
         <v>26</v>
       </c>
       <c r="S6" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T6" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T6" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V6" s="11"/>
       <c r="W6" s="11"/>
@@ -1910,70 +2125,72 @@
         <v>26</v>
       </c>
       <c r="Y6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:25">
       <c r="A7" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T7" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T7" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
@@ -1981,143 +2198,145 @@
         <v>26</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
       <c r="X8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I9" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T9" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T9" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
@@ -2125,72 +2344,72 @@
         <v>26</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T10" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="V10" s="11"/>
       <c r="W10" s="11"/>
@@ -2198,70 +2417,72 @@
         <v>26</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I11" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T11" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T11" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V11" s="11"/>
       <c r="W11" s="11"/>
@@ -2269,291 +2490,310 @@
         <v>26</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:25">
       <c r="A12" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T12" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T12" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V12" s="11"/>
       <c r="W12" s="11"/>
       <c r="X12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>26</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R13" s="10" t="s">
         <v>26</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T13" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="T13" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="U13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V13" s="11"/>
       <c r="W13" s="11"/>
       <c r="X13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:25">
       <c r="A14" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>26</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T14" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V14" s="11"/>
       <c r="W14" s="11"/>
       <c r="X14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="I15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S15" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="T15" s="10"/>
+      <c r="T15" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="U15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V15" s="11"/>
       <c r="W15" s="11"/>
       <c r="X15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="5:18">
+      <c r="E17" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q17" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="R17" s="13" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2571,47 +2811,47 @@
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X15:Y15">
+  <conditionalFormatting sqref="X15">
     <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X15:Y15">
+  <conditionalFormatting sqref="X15">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X15:Y15">
+  <conditionalFormatting sqref="X15">
     <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:U15">
+  <conditionalFormatting sqref="B15 H15:J15 S15:U15">
     <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:U15">
+  <conditionalFormatting sqref="B15 H15:J15 S15:U15">
     <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:U15">
+  <conditionalFormatting sqref="B15 H15:J15 S15:U15">
     <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:Y14">
+  <conditionalFormatting sqref="B3:Y14 C15:G15 K15:R15 Y15">
     <cfRule type="cellIs" dxfId="8" priority="9" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C14">
+  <conditionalFormatting sqref="C3:C15">
     <cfRule type="cellIs" dxfId="9" priority="10" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:Y14">
+  <conditionalFormatting sqref="B3:Y14 C15:G15 K15:R15 Y15">
     <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
       <formula>N</formula>
     </cfRule>
@@ -2619,7 +2859,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2628,14 +2868,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2654,7 +2894,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2664,25 +2904,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -2694,7 +2934,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2705,14 +2945,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2731,7 +2971,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2763,7 +3003,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2774,14 +3014,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2800,7 +3040,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2810,55 +3050,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -2870,7 +3110,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2881,14 +3121,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2907,7 +3147,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2917,19 +3157,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -2941,7 +3181,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2952,14 +3192,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2978,7 +3218,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2988,18 +3228,18 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="2:2">
@@ -3043,7 +3283,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3054,14 +3294,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3080,7 +3320,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3090,55 +3330,69 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B5" s="10"/>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
+        <v>48</v>
+      </c>
+      <c r="B6" s="10"/>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
+        <v>49</v>
+      </c>
+      <c r="B7" s="10"/>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
+        <v>50</v>
+      </c>
+      <c r="B8" s="10"/>
+    </row>
+    <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>49</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="B9" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B9">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B9">
+    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3149,14 +3403,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3175,7 +3429,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3195,7 +3449,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3206,14 +3460,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3232,7 +3486,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3242,137 +3496,137 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="10"/>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B12" s="10"/>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B13" s="10"/>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B14" s="10"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B15" s="10"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B16" s="10"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B17" s="10"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B19" s="10"/>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B21" s="10"/>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B22" s="10"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B23" s="10"/>
       <c r="D23" s="10"/>
@@ -3383,29 +3637,29 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="D23">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D23">
-    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B23">
-    <cfRule type="cellIs" dxfId="19" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B23">
-    <cfRule type="cellIs" dxfId="20" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3416,14 +3670,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3442,7 +3696,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3452,37 +3706,37 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B8" s="10"/>
     </row>
@@ -3494,7 +3748,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3505,14 +3759,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3523,7 +3777,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
@@ -3531,7 +3785,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3541,25 +3795,32 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="10"/>
+        <v>78</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="10"/>
-    </row>
-    <row r="5" spans="1:2">
+        <v>79</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="10"/>
+        <v>80</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -3568,10 +3829,20 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B6">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B6">
+    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3582,14 +3853,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3600,7 +3871,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
@@ -3608,7 +3879,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3618,49 +3889,90 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="10"/>
+        <v>82</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" s="10"/>
+        <v>84</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="10"/>
+        <v>85</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7" s="10"/>
-    </row>
-    <row r="8" spans="1:2">
+        <v>86</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B8" s="10"/>
+      <c r="D8" s="10"/>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="10"/>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="D8">
+    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D8">
+    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B10">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B10">
+    <cfRule type="cellIs" dxfId="28" priority="4" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3671,14 +3983,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3697,7 +4009,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3707,31 +4019,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -3743,7 +4055,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1773323801" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3754,14 +4066,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1773323801" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773323801" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Fixed enum/error set array
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1776900014" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1776900014" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1776900014" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1776900014"/>
+      <pm:revision xmlns:pm="smNativeData" day="1776932651" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1776932651" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1776932651" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1776932651"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="112">
   <si>
     <t>Context</t>
   </si>
@@ -115,12 +115,12 @@
     <t>As static variable</t>
   </si>
   <si>
+    <t>Y</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>?</t>
   </si>
   <si>
@@ -161,6 +161,9 @@
   </si>
   <si>
     <t>leak</t>
+  </si>
+  <si>
+    <t>segfault</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -397,7 +400,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776932651" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -412,7 +415,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776932651" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -427,7 +430,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776932651" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -443,7 +446,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776900014" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776932651" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -452,7 +455,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -465,7 +468,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -476,7 +479,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -487,7 +490,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -498,7 +501,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -509,7 +512,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -520,13 +523,24 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -542,7 +556,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776900014"/>
+          <pm:border xmlns:pm="smNativeData" id="1776932651"/>
         </ext>
       </extLst>
     </border>
@@ -561,7 +575,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776900014">
+          <pm:border xmlns:pm="smNativeData" id="1776932651">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -583,7 +597,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776900014">
+          <pm:border xmlns:pm="smNativeData" id="1776932651">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -607,7 +621,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776900014">
+          <pm:border xmlns:pm="smNativeData" id="1776932651">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -631,7 +645,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776900014">
+          <pm:border xmlns:pm="smNativeData" id="1776932651">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -655,7 +669,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776900014"/>
+          <pm:border xmlns:pm="smNativeData" id="1776932651"/>
         </ext>
       </extLst>
     </border>
@@ -674,7 +688,26 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776900014"/>
+          <pm:border xmlns:pm="smNativeData" id="1776932651"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1776932651"/>
         </ext>
       </extLst>
     </border>
@@ -687,7 +720,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -718,6 +751,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -733,7 +769,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -746,7 +782,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -757,7 +793,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -770,7 +806,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -781,7 +817,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -794,7 +830,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -805,7 +841,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -818,7 +854,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -829,7 +865,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -842,7 +878,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -853,7 +889,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -866,7 +902,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -877,7 +913,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -890,7 +926,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -901,7 +937,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -914,7 +950,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -925,7 +961,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -938,7 +974,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -949,7 +985,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -962,7 +998,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -973,7 +1009,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -986,7 +1022,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -997,7 +1033,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1010,7 +1046,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1021,7 +1057,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1034,7 +1070,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1045,7 +1081,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1058,7 +1094,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1069,7 +1105,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1082,7 +1118,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1093,7 +1129,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1106,7 +1142,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1117,7 +1153,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1130,7 +1166,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1141,7 +1177,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1154,7 +1190,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1165,7 +1201,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1178,7 +1214,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1189,7 +1225,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1202,7 +1238,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1213,7 +1249,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1226,7 +1262,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1237,7 +1273,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1250,7 +1286,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1261,7 +1297,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1274,7 +1310,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1285,7 +1321,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1298,7 +1334,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1309,7 +1345,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1322,7 +1358,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1333,7 +1369,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1346,7 +1382,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1357,7 +1393,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1370,7 +1406,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1381,7 +1417,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1394,7 +1430,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1405,7 +1441,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776900014" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1776932651" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1418,7 +1454,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776900014" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1776932651" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1428,10 +1464,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1776900014" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1776932651" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1776900014" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1776932651" count="6">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -1704,30 +1740,30 @@
   <sheetFormatPr baseColWidth="7" defaultColWidth="8.544643" defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="22.151786" customWidth="1" style="0"/>
-    <col min="2" max="2" width="5.276786" customWidth="1" style="0"/>
-    <col min="3" max="3" width="5.142857" customWidth="1" style="0"/>
-    <col min="4" max="4" width="5.000000" customWidth="1" style="0"/>
-    <col min="5" max="5" width="9.571429" customWidth="1" style="0"/>
-    <col min="6" max="6" width="3.428571" customWidth="1" style="0"/>
-    <col min="7" max="7" width="5.428571" customWidth="1" style="0"/>
-    <col min="8" max="8" width="7.571429" customWidth="1" style="0"/>
-    <col min="9" max="9" width="5.696429" customWidth="1" style="0"/>
-    <col min="10" max="10" width="6.142857" customWidth="1" style="0"/>
-    <col min="11" max="11" width="14.848214" customWidth="1" style="0"/>
-    <col min="12" max="12" width="12.705357" customWidth="1" style="0"/>
-    <col min="13" max="13" width="10.428571" customWidth="1" style="0"/>
-    <col min="14" max="14" width="4.696429" customWidth="1" style="0"/>
-    <col min="15" max="15" width="8.696429" customWidth="1" style="0"/>
-    <col min="16" max="16" width="10.571429" customWidth="1" style="0"/>
-    <col min="17" max="17" width="8.142857" customWidth="1" style="0"/>
-    <col min="18" max="18" width="6.000000" customWidth="1" style="0"/>
-    <col min="19" max="19" width="6.276786" customWidth="1" style="0"/>
-    <col min="20" max="20" width="3.142857" customWidth="1" style="0"/>
-    <col min="21" max="21" width="8.000000" customWidth="1" style="0"/>
-    <col min="22" max="22" width="6.571429" customWidth="1" style="0"/>
-    <col min="23" max="23" width="10.000000" customWidth="1" style="0"/>
-    <col min="24" max="24" width="6.848214" customWidth="1" style="0"/>
-    <col min="25" max="25" width="11.571429" customWidth="1" style="0"/>
+    <col min="2" max="2" width="4.660714" customWidth="1" style="0"/>
+    <col min="3" max="3" width="4.437500" customWidth="1" style="0"/>
+    <col min="4" max="4" width="4.392857" customWidth="1" style="0"/>
+    <col min="5" max="5" width="8.562500" customWidth="1" style="0"/>
+    <col min="6" max="6" width="2.991071" customWidth="1" style="0"/>
+    <col min="7" max="7" width="4.785714" customWidth="1" style="0"/>
+    <col min="8" max="8" width="6.660714" customWidth="1" style="0"/>
+    <col min="9" max="9" width="7.151786" customWidth="1" style="0"/>
+    <col min="10" max="10" width="5.580357" customWidth="1" style="0"/>
+    <col min="11" max="11" width="13.125000" customWidth="1" style="0"/>
+    <col min="12" max="12" width="11.330357" customWidth="1" style="0"/>
+    <col min="13" max="13" width="9.196429" customWidth="1" style="0"/>
+    <col min="14" max="14" width="4.000000" customWidth="1" style="0"/>
+    <col min="15" max="15" width="7.705357" customWidth="1" style="0"/>
+    <col min="16" max="16" width="9.669643" customWidth="1" style="0"/>
+    <col min="17" max="17" width="7.392857" customWidth="1" style="0"/>
+    <col min="18" max="18" width="5.401786" customWidth="1" style="0"/>
+    <col min="19" max="19" width="5.616071" customWidth="1" style="0"/>
+    <col min="20" max="20" width="2.741071" customWidth="1" style="0"/>
+    <col min="21" max="21" width="7.125000" customWidth="1" style="0"/>
+    <col min="22" max="22" width="5.875000" customWidth="1" style="0"/>
+    <col min="23" max="23" width="8.937500" customWidth="1" style="0"/>
+    <col min="24" max="24" width="6.107143" customWidth="1" style="0"/>
+    <col min="25" max="25" width="10.375000" customWidth="1" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1844,61 +1880,61 @@
         <v>26</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="I3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="K3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P3" s="10" t="s">
         <v>26</v>
       </c>
       <c r="Q3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T3" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V3" s="11"/>
       <c r="W3" s="11"/>
@@ -1906,7 +1942,7 @@
         <v>26</v>
       </c>
       <c r="Y3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1914,72 +1950,72 @@
         <v>29</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="K4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T4" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V4" s="11"/>
       <c r="W4" s="11"/>
       <c r="X4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1987,72 +2023,72 @@
         <v>30</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="F5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T5" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V5" s="11"/>
       <c r="W5" s="11"/>
       <c r="X5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -2063,34 +2099,34 @@
         <v>28</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I6" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M6" s="10" t="s">
         <v>26</v>
@@ -2099,10 +2135,10 @@
         <v>26</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q6" s="10" t="s">
         <v>26</v>
@@ -2111,13 +2147,13 @@
         <v>26</v>
       </c>
       <c r="S6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T6" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V6" s="11"/>
       <c r="W6" s="11"/>
@@ -2125,7 +2161,7 @@
         <v>26</v>
       </c>
       <c r="Y6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -2133,64 +2169,64 @@
         <v>32</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="I7" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T7" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
@@ -2198,7 +2234,7 @@
         <v>26</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -2206,61 +2242,61 @@
         <v>33</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>28</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="U8" s="10" t="s">
         <v>28</v>
@@ -2268,10 +2304,10 @@
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
       <c r="X8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -2279,64 +2315,64 @@
         <v>34</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I9" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T9" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
@@ -2344,7 +2380,7 @@
         <v>26</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -2352,58 +2388,58 @@
         <v>35</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T10" s="10" t="s">
         <v>28</v>
@@ -2417,7 +2453,7 @@
         <v>26</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -2425,64 +2461,64 @@
         <v>36</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="I11" s="10" t="s">
         <v>26</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T11" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V11" s="11"/>
       <c r="W11" s="11"/>
@@ -2490,7 +2526,7 @@
         <v>26</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -2498,72 +2534,72 @@
         <v>37</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="I12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T12" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V12" s="11"/>
       <c r="W12" s="11"/>
       <c r="X12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -2571,72 +2607,72 @@
         <v>38</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="I13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="O13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R13" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="L13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="N13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="O13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="R13" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="S13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T13" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V13" s="11"/>
       <c r="W13" s="11"/>
       <c r="X13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -2644,72 +2680,72 @@
         <v>39</v>
       </c>
       <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="I14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="T14" s="10" t="s">
         <v>28</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V14" s="11"/>
       <c r="W14" s="11"/>
       <c r="X14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -2717,76 +2753,82 @@
         <v>40</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="J15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="K15" s="10" t="s">
+      <c r="T15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="L15" s="10" t="s">
+      <c r="U15" s="10" t="s">
         <v>27</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="N15" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="O15" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="P15" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q15" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="R15" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="S15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="U15" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="V15" s="11"/>
       <c r="W15" s="11"/>
       <c r="X15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="5:18">
       <c r="E17" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="P17" s="13" t="s">
         <v>41</v>
       </c>
       <c r="Q17" s="13" t="s">
@@ -2859,7 +2901,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2868,14 +2910,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2894,7 +2936,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2904,25 +2946,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -2934,7 +2976,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2945,14 +2987,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2971,7 +3013,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3003,7 +3045,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3014,14 +3056,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3040,7 +3082,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3050,55 +3092,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3110,7 +3152,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3121,14 +3163,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3147,7 +3189,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3157,19 +3199,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3181,7 +3223,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3192,14 +3234,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3218,7 +3260,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3228,18 +3270,18 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="2:2">
@@ -3283,7 +3325,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3294,14 +3336,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3320,7 +3362,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3330,47 +3372,47 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B9" s="10"/>
     </row>
@@ -3392,7 +3434,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3403,14 +3445,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3429,7 +3471,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3449,7 +3491,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3460,14 +3502,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3486,7 +3528,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3496,137 +3538,137 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11" s="10"/>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="10"/>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B13" s="10"/>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="10"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B15" s="10"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B16" s="10"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B17" s="10"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B19" s="10"/>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B21" s="10"/>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B22" s="10"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B23" s="10"/>
       <c r="D23" s="10"/>
@@ -3659,7 +3701,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3670,14 +3712,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3696,7 +3738,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3706,37 +3748,37 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B8" s="10"/>
     </row>
@@ -3748,7 +3790,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3759,14 +3801,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3785,7 +3827,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3795,32 +3837,32 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -3842,7 +3884,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3853,14 +3895,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3879,7 +3921,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3889,58 +3931,58 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -3972,7 +4014,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3983,14 +4025,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4009,7 +4051,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -4019,31 +4061,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -4055,7 +4097,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776900014" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776932651" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4066,14 +4108,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776900014" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776932651" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776900014" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776932651" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Fixed leak from error set (#888)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1776978388" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1776978388" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1776978388" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1776978388"/>
+      <pm:revision xmlns:pm="smNativeData" day="1777080888" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1777080888" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1777080888" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1777080888"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="110">
   <si>
     <t>Context</t>
   </si>
@@ -158,12 +158,6 @@
   </si>
   <si>
     <t>Constructor</t>
-  </si>
-  <si>
-    <t>leak</t>
-  </si>
-  <si>
-    <t>segfault</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -400,7 +394,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776978388" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -415,7 +409,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776978388" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -430,7 +424,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776978388" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -446,7 +440,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776978388" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -468,7 +462,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -479,7 +473,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -490,7 +484,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -501,7 +495,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -512,7 +506,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF9E"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -523,7 +528,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -534,18 +539,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF9E"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -567,7 +561,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388"/>
+          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
         </ext>
       </extLst>
     </border>
@@ -586,7 +580,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388">
+          <pm:border xmlns:pm="smNativeData" id="1777080888">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -608,7 +602,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388">
+          <pm:border xmlns:pm="smNativeData" id="1777080888">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -632,7 +626,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388">
+          <pm:border xmlns:pm="smNativeData" id="1777080888">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -656,7 +650,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388">
+          <pm:border xmlns:pm="smNativeData" id="1777080888">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -680,7 +674,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388"/>
+          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
         </ext>
       </extLst>
     </border>
@@ -699,7 +693,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388"/>
+          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
         </ext>
       </extLst>
     </border>
@@ -718,7 +712,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388"/>
+          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
         </ext>
       </extLst>
     </border>
@@ -737,7 +731,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776978388"/>
+          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
         </ext>
       </extLst>
     </border>
@@ -750,7 +744,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -781,10 +775,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -802,7 +793,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -815,7 +806,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -826,7 +817,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -839,7 +830,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -850,7 +841,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -863,7 +854,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -874,7 +865,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -887,7 +878,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -898,7 +889,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -911,7 +902,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -922,7 +913,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -935,7 +926,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -946,7 +937,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -959,7 +950,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -970,7 +961,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -983,7 +974,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -994,7 +985,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1007,7 +998,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1018,7 +1009,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1031,7 +1022,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1042,7 +1033,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1055,7 +1046,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1066,7 +1057,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1079,7 +1070,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1090,7 +1081,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1103,7 +1094,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1114,7 +1105,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1127,7 +1118,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1138,7 +1129,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1151,7 +1142,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1162,7 +1153,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1175,7 +1166,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1186,7 +1177,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1199,7 +1190,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1210,7 +1201,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1223,7 +1214,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1234,7 +1225,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1247,7 +1238,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1258,7 +1249,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1271,7 +1262,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1282,7 +1273,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1295,7 +1286,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1306,7 +1297,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1319,7 +1310,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1330,7 +1321,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1343,7 +1334,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1354,7 +1345,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1367,7 +1358,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1378,7 +1369,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1391,7 +1382,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1402,7 +1393,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1415,7 +1406,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1426,7 +1417,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1439,7 +1430,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1450,7 +1441,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1463,7 +1454,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1474,7 +1465,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1776978388" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1487,7 +1478,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1776978388" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1497,16 +1488,17 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1776978388" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1777080888" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1776978388" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1777080888" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
         <pm:color name="Color 27" rgb="92D050"/>
         <pm:color name="Color 28" rgb="808080"/>
         <pm:color name="Color 29" rgb="FFB3B3"/>
+        <pm:color name="Color 30" rgb="FFFF9E"/>
       </pm:colors>
     </ext>
   </extLst>
@@ -1773,7 +1765,7 @@
   <sheetFormatPr baseColWidth="7" defaultColWidth="8.544643" defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="22.151786" customWidth="1" style="0"/>
-    <col min="2" max="2" width="4.660714" customWidth="1" style="0"/>
+    <col min="2" max="2" width="7.151786" customWidth="1" style="0"/>
     <col min="3" max="3" width="4.437500" customWidth="1" style="0"/>
     <col min="4" max="4" width="4.392857" customWidth="1" style="0"/>
     <col min="5" max="5" width="8.562500" customWidth="1" style="0"/>
@@ -1783,12 +1775,11 @@
     <col min="11" max="11" width="13.125000" customWidth="1" style="0"/>
     <col min="12" max="12" width="11.330357" customWidth="1" style="0"/>
     <col min="13" max="13" width="9.196429" customWidth="1" style="0"/>
-    <col min="14" max="14" width="4.000000" customWidth="1" style="0"/>
+    <col min="14" max="14" width="7.151786" customWidth="1" style="0"/>
     <col min="15" max="15" width="7.705357" customWidth="1" style="0"/>
     <col min="16" max="16" width="9.669643" customWidth="1" style="0"/>
     <col min="17" max="17" width="7.392857" customWidth="1" style="0"/>
-    <col min="18" max="18" width="5.401786" customWidth="1" style="0"/>
-    <col min="19" max="19" width="7.151786" customWidth="1" style="0"/>
+    <col min="18" max="19" width="7.151786" customWidth="1" style="0"/>
     <col min="20" max="20" width="2.741071" customWidth="1" style="0"/>
     <col min="21" max="21" width="7.125000" customWidth="1" style="0"/>
     <col min="22" max="22" width="5.875000" customWidth="1" style="0"/>
@@ -2801,7 +2792,7 @@
       <c r="G15" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="10" t="s">
         <v>26</v>
       </c>
       <c r="I15" s="10" t="s">
@@ -2852,34 +2843,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="5:24">
-      <c r="E17" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="I17" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="J17" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="P17" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q17" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="R17" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="S17" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="X17" s="13" t="s">
-        <v>42</v>
-      </c>
+    <row r="17" spans="2:24">
+      <c r="B17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="P17" s="13"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="13"/>
+      <c r="S17" s="13"/>
+      <c r="X17" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2944,7 +2921,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2953,14 +2930,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2979,7 +2956,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2989,25 +2966,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -3019,7 +2996,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3030,14 +3007,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3056,7 +3033,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3088,7 +3065,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3099,14 +3076,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3125,7 +3102,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3135,55 +3112,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3195,7 +3172,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3206,14 +3183,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3232,7 +3209,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3242,19 +3219,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3266,7 +3243,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3277,14 +3254,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3303,7 +3280,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3313,7 +3290,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3321,7 +3298,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3368,7 +3345,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3379,14 +3356,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3405,7 +3382,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3415,7 +3392,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3423,7 +3400,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3431,31 +3408,31 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B9" s="10"/>
     </row>
@@ -3477,7 +3454,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3488,14 +3465,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3514,7 +3491,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3534,7 +3511,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3545,14 +3522,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3571,7 +3548,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3581,7 +3558,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3589,7 +3566,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>28</v>
@@ -3597,31 +3574,31 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -3629,55 +3606,55 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B11" s="10"/>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B12" s="10"/>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B13" s="10"/>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B14" s="10"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B15" s="10"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B16" s="10"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B17" s="10"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>28</v>
@@ -3685,13 +3662,13 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B19" s="10"/>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>26</v>
@@ -3699,19 +3676,19 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B21" s="10"/>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B22" s="10"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B23" s="10"/>
       <c r="D23" s="10"/>
@@ -3744,7 +3721,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3755,14 +3732,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3781,7 +3758,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3791,37 +3768,37 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8" s="10"/>
     </row>
@@ -3833,7 +3810,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3844,14 +3821,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3870,7 +3847,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3880,7 +3857,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3888,7 +3865,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3896,7 +3873,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>28</v>
@@ -3905,7 +3882,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -3927,7 +3904,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3938,14 +3915,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3964,7 +3941,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3974,7 +3951,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>28</v>
@@ -3982,13 +3959,13 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3996,7 +3973,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>28</v>
@@ -4004,7 +3981,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4012,20 +3989,20 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -4057,7 +4034,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4068,14 +4045,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4094,7 +4071,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -4104,31 +4081,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -4140,7 +4117,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776978388" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4151,14 +4128,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776978388" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776978388" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added C pointer handling and null pointer check
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="0" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="592"/>
+    <workbookView activeTab="4" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="592"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1777080888" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1777080888" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1777080888" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1777080888"/>
+      <pm:revision xmlns:pm="smNativeData" day="1777243520" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1777243520" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1777243520" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1777243520"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="121">
   <si>
     <t>Context</t>
   </si>
@@ -205,27 +205,12 @@
     <t>Print slice of slices</t>
   </si>
   <si>
-    <t>Accept typed array</t>
-  </si>
-  <si>
     <t>Return bool vector</t>
   </si>
   <si>
-    <t>Handle misaligned pointer</t>
-  </si>
-  <si>
-    <t>Handle misaligned aliased pointer</t>
-  </si>
-  <si>
     <t>Allocate slice of structs</t>
   </si>
   <si>
-    <t>Clear pointers</t>
-  </si>
-  <si>
-    <t>Clear pointer array</t>
-  </si>
-  <si>
     <t>Attach getters/setters</t>
   </si>
   <si>
@@ -253,6 +238,51 @@
     <t>Return const pointer</t>
   </si>
   <si>
+    <t>Accept multiple pointers</t>
+  </si>
+  <si>
+    <t>Accept C pointers</t>
+  </si>
+  <si>
+    <t>Return C pointers</t>
+  </si>
+  <si>
+    <t>Modify a pointer target</t>
+  </si>
+  <si>
+    <t>Call functions</t>
+  </si>
+  <si>
+    <t>Call variadic functions</t>
+  </si>
+  <si>
+    <t>Pass unsigned in to variadic function</t>
+  </si>
+  <si>
+    <t>Write to file using fwrite</t>
+  </si>
+  <si>
+    <t>Read from file using fread</t>
+  </si>
+  <si>
+    <t>Call printf</t>
+  </si>
+  <si>
+    <t>Call fprintf</t>
+  </si>
+  <si>
+    <t>Call sprintf</t>
+  </si>
+  <si>
+    <t>Call snprintf</t>
+  </si>
+  <si>
+    <t>Handle immediate promise fulfillment</t>
+  </si>
+  <si>
+    <t>Apply transform to return value</t>
+  </si>
+  <si>
     <t>Free function thunk</t>
   </si>
   <si>
@@ -278,6 +308,9 @@
   </si>
   <si>
     <t>Return allocator</t>
+  </si>
+  <si>
+    <t>leak</t>
   </si>
   <si>
     <t>Thread creation</t>
@@ -394,7 +427,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -409,7 +442,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -424,7 +457,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -440,7 +473,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777080888" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -449,7 +482,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -462,7 +495,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -473,7 +506,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -484,7 +517,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -495,7 +528,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -506,7 +539,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -517,7 +550,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -528,24 +561,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFB3B3"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -561,7 +583,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
+          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
         </ext>
       </extLst>
     </border>
@@ -580,7 +602,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888">
+          <pm:border xmlns:pm="smNativeData" id="1777243520">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -602,7 +624,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888">
+          <pm:border xmlns:pm="smNativeData" id="1777243520">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -626,7 +648,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888">
+          <pm:border xmlns:pm="smNativeData" id="1777243520">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -650,7 +672,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888">
+          <pm:border xmlns:pm="smNativeData" id="1777243520">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -674,7 +696,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
+          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
         </ext>
       </extLst>
     </border>
@@ -693,7 +715,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
+          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
         </ext>
       </extLst>
     </border>
@@ -712,26 +734,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777080888"/>
+          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
         </ext>
       </extLst>
     </border>
@@ -787,13 +790,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="29">
+  <dxfs count="31">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -806,7 +809,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -817,7 +820,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -830,7 +833,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -841,7 +844,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -854,7 +857,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -865,7 +868,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -878,7 +881,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -889,7 +892,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -902,7 +905,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -913,7 +916,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -926,7 +929,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -937,7 +940,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -950,7 +953,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -961,7 +964,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -974,7 +977,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -985,7 +988,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -998,7 +1001,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1009,7 +1012,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1022,7 +1025,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1033,7 +1036,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1046,7 +1049,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1057,7 +1060,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1070,7 +1073,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1081,7 +1084,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1094,7 +1097,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1105,7 +1108,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1118,7 +1121,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1129,7 +1132,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1142,7 +1145,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1153,7 +1156,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1166,7 +1169,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1177,7 +1180,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1190,7 +1193,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1201,7 +1204,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1214,7 +1217,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1225,7 +1228,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1238,7 +1241,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1249,7 +1252,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1262,7 +1265,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1273,7 +1276,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1286,7 +1289,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1297,7 +1300,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1310,7 +1313,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1321,7 +1324,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1334,7 +1337,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1345,7 +1348,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1358,7 +1361,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1369,7 +1372,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1382,7 +1385,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1393,7 +1396,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1406,7 +1409,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1417,7 +1420,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1430,7 +1433,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1441,7 +1444,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1454,7 +1457,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1465,7 +1468,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777080888" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1478,7 +1481,55 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777080888" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1488,10 +1539,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1777080888" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1777243520" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1777080888" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1777243520" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -2921,7 +2972,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2930,14 +2981,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2966,25 +3017,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -2996,7 +3047,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3007,14 +3058,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3065,7 +3116,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3076,14 +3127,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3112,55 +3163,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3172,7 +3223,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3183,14 +3234,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3219,19 +3270,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3243,7 +3294,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3254,14 +3305,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3345,7 +3396,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3356,14 +3407,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3454,7 +3505,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3465,14 +3516,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3511,7 +3562,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3522,14 +3573,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3540,7 +3591,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="35.062500" customWidth="1" style="0"/>
@@ -3569,32 +3620,40 @@
         <v>52</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="10"/>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="10"/>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
@@ -3608,83 +3667,104 @@
       <c r="A10" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="10"/>
+      <c r="B11" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="10"/>
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="10"/>
+      <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B15" s="10"/>
+      <c r="B15" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B17" s="10"/>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="B17" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="9" t="s">
         <v>66</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="D18" s="10"/>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="10"/>
-    </row>
-    <row r="20" spans="1:2">
+      <c r="B19" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="10"/>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="B20" s="10"/>
+      <c r="D20" s="10"/>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
         <v>69</v>
       </c>
       <c r="B21" s="10"/>
-    </row>
-    <row r="22" spans="1:2">
+      <c r="D21" s="10"/>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="9" t="s">
         <v>70</v>
       </c>
       <c r="B22" s="10"/>
+      <c r="D22" s="10"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
@@ -3692,36 +3772,116 @@
       </c>
       <c r="B23" s="10"/>
       <c r="D23" s="10"/>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="10"/>
+      <c r="D24" s="10"/>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="10"/>
+      <c r="D25" s="10"/>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B26" s="10"/>
+      <c r="D26" s="10"/>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="10"/>
+      <c r="D27" s="10"/>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" s="10"/>
+      <c r="D28" s="10"/>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="10"/>
+      <c r="D29" s="10"/>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" s="10"/>
+      <c r="D30" s="10"/>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" s="10"/>
+      <c r="D31" s="10"/>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B32" s="10"/>
+      <c r="D32" s="10"/>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B33" s="10"/>
+      <c r="D33" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="D23">
+  <conditionalFormatting sqref="B19:B33">
     <cfRule type="cellIs" dxfId="19" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D23">
+  <conditionalFormatting sqref="B19:B33">
     <cfRule type="cellIs" dxfId="20" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B23">
+  <conditionalFormatting sqref="D18">
     <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B23">
+  <conditionalFormatting sqref="D18">
     <cfRule type="cellIs" dxfId="22" priority="4" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B18">
+    <cfRule type="cellIs" dxfId="23" priority="5" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B18">
+    <cfRule type="cellIs" dxfId="24" priority="6" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3732,14 +3892,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3768,31 +3928,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -3810,7 +3970,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3821,14 +3981,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3839,7 +3999,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
@@ -3857,7 +4017,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3865,7 +4025,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3873,18 +4033,23 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B6" s="10"/>
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" s="13" t="s">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3892,19 +4057,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B6">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B6">
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3915,14 +4080,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3951,7 +4116,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>28</v>
@@ -3959,13 +4124,13 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3973,7 +4138,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>28</v>
@@ -3981,7 +4146,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -3989,20 +4154,20 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="B8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -4012,29 +4177,29 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="D8">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D8">
-    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="28" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4045,14 +4210,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4081,31 +4246,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -4117,7 +4282,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777080888" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4128,14 +4293,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777080888" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777080888" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added more tests (#908)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1777243520" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1777243520" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1777243520" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1777243520"/>
+      <pm:revision xmlns:pm="smNativeData" day="1777486352" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1777486352" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1777486352" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1777486352"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="123">
   <si>
     <t>Context</t>
   </si>
@@ -241,16 +241,25 @@
     <t>Accept multiple pointers</t>
   </si>
   <si>
+    <t>segfault</t>
+  </si>
+  <si>
     <t>Accept C pointers</t>
   </si>
   <si>
+    <t>Return multiple pointers</t>
+  </si>
+  <si>
     <t>Return C pointers</t>
   </si>
   <si>
     <t>Modify a pointer target</t>
   </si>
   <si>
-    <t>Call functions</t>
+    <t>Call C functions</t>
+  </si>
+  <si>
+    <t>leak</t>
   </si>
   <si>
     <t>Call variadic functions</t>
@@ -308,9 +317,6 @@
   </si>
   <si>
     <t>Return allocator</t>
-  </si>
-  <si>
-    <t>leak</t>
   </si>
   <si>
     <t>Thread creation</t>
@@ -427,7 +433,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -442,7 +448,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -457,7 +463,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -473,7 +479,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777243520" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -482,7 +488,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -495,7 +501,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -506,7 +512,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -517,7 +523,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -528,7 +534,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -539,7 +545,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -550,7 +556,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -561,13 +567,35 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -583,7 +611,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
+          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
         </ext>
       </extLst>
     </border>
@@ -602,7 +630,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520">
+          <pm:border xmlns:pm="smNativeData" id="1777486352">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -624,7 +652,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520">
+          <pm:border xmlns:pm="smNativeData" id="1777486352">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -648,7 +676,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520">
+          <pm:border xmlns:pm="smNativeData" id="1777486352">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -672,7 +700,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520">
+          <pm:border xmlns:pm="smNativeData" id="1777486352">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -696,7 +724,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
+          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
         </ext>
       </extLst>
     </border>
@@ -715,7 +743,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
+          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
         </ext>
       </extLst>
     </border>
@@ -734,7 +762,45 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777243520"/>
+          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
         </ext>
       </extLst>
     </border>
@@ -796,7 +862,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -809,7 +875,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -820,7 +886,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -833,7 +899,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -844,7 +910,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -857,7 +923,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -868,7 +934,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -881,7 +947,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -892,7 +958,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -905,7 +971,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -916,7 +982,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -929,7 +995,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -940,7 +1006,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -953,7 +1019,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -964,7 +1030,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -977,7 +1043,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -988,7 +1054,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1001,7 +1067,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1012,7 +1078,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1025,7 +1091,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1036,7 +1102,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1049,7 +1115,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1060,7 +1126,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1073,7 +1139,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1084,7 +1150,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1097,7 +1163,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1108,7 +1174,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1121,7 +1187,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1132,7 +1198,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1145,7 +1211,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1156,7 +1222,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1169,7 +1235,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1180,7 +1246,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1193,7 +1259,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1204,7 +1270,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1217,7 +1283,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1228,7 +1294,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1241,7 +1307,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1252,7 +1318,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1265,7 +1331,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1276,7 +1342,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1289,7 +1355,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1300,7 +1366,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1313,7 +1379,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1324,7 +1390,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1337,7 +1403,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1348,7 +1414,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1361,7 +1427,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1372,7 +1438,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1385,7 +1451,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1396,7 +1462,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1409,7 +1475,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1420,7 +1486,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1433,7 +1499,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1444,7 +1510,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1457,7 +1523,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1468,7 +1534,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1481,7 +1547,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1492,7 +1558,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1505,7 +1571,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1516,7 +1582,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777243520" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1529,7 +1595,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777243520" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1539,10 +1605,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1777243520" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1777486352" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1777243520" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1777486352" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -2972,7 +3038,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2981,14 +3047,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3017,25 +3083,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -3047,7 +3113,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3058,14 +3124,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3116,7 +3182,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3127,14 +3193,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3163,55 +3229,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3223,7 +3289,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3234,14 +3300,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3270,19 +3336,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3294,7 +3360,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3305,14 +3371,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3396,7 +3462,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3407,14 +3473,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3505,7 +3571,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3516,14 +3582,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3562,7 +3628,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3573,14 +3639,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3591,7 +3657,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="35.062500" customWidth="1" style="0"/>
@@ -3741,119 +3807,174 @@
         <v>67</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="D20" s="10"/>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B21" s="10"/>
-      <c r="D21" s="10"/>
+        <v>70</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B22" s="10"/>
-      <c r="D22" s="10"/>
+        <v>71</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="10"/>
-      <c r="D23" s="10"/>
+        <v>72</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B24" s="10"/>
-      <c r="D24" s="10"/>
+        <v>73</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B25" s="10"/>
-      <c r="D25" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="D26" s="10"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B27" s="10"/>
-      <c r="D27" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B28" s="10"/>
       <c r="D28" s="10"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B29" s="10"/>
-      <c r="D29" s="10"/>
+        <v>79</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B30" s="10"/>
-      <c r="D30" s="10"/>
+        <v>80</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B31" s="10"/>
       <c r="D31" s="10"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B32" s="10"/>
       <c r="D32" s="10"/>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B33" s="10"/>
+        <v>83</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="D33" s="10"/>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B19:B33">
+  <conditionalFormatting sqref="B19:B34">
     <cfRule type="cellIs" dxfId="19" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B19:B33">
+  <conditionalFormatting sqref="B19:B34">
     <cfRule type="cellIs" dxfId="20" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
@@ -3881,7 +4002,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3892,14 +4013,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3928,31 +4049,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -3970,7 +4091,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3981,14 +4102,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4017,7 +4138,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4025,7 +4146,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4033,7 +4154,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4042,13 +4163,13 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="8" spans="2:2">
       <c r="B8" s="13" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -4069,7 +4190,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4080,14 +4201,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4116,7 +4237,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>28</v>
@@ -4124,13 +4245,13 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4138,7 +4259,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>28</v>
@@ -4146,7 +4267,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4154,20 +4275,20 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -4199,7 +4320,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4210,14 +4331,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4246,31 +4367,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -4282,7 +4403,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777243520" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4293,14 +4414,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777243520" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777243520" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Fixed recursion crash (#899)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1777486352" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1777486352" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1777486352" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1777486352"/>
+      <pm:revision xmlns:pm="smNativeData" day="1777560623" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1777560623" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1777560623" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1777560623"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="123">
   <si>
     <t>Context</t>
   </si>
@@ -235,6 +235,9 @@
     <t>Handle recursive structure</t>
   </si>
   <si>
+    <t>leak</t>
+  </si>
+  <si>
     <t>Return const pointer</t>
   </si>
   <si>
@@ -257,9 +260,6 @@
   </si>
   <si>
     <t>Call C functions</t>
-  </si>
-  <si>
-    <t>leak</t>
   </si>
   <si>
     <t>Call variadic functions</t>
@@ -433,7 +433,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -448,7 +448,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -463,7 +463,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -479,7 +479,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777486352" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -488,7 +488,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -501,7 +501,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -512,7 +512,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -523,7 +523,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -534,7 +534,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -545,7 +545,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -556,7 +556,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -567,7 +567,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -578,24 +578,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -611,7 +600,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
+          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
         </ext>
       </extLst>
     </border>
@@ -630,7 +619,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352">
+          <pm:border xmlns:pm="smNativeData" id="1777560623">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -652,7 +641,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352">
+          <pm:border xmlns:pm="smNativeData" id="1777560623">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -676,7 +665,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352">
+          <pm:border xmlns:pm="smNativeData" id="1777560623">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -700,7 +689,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352">
+          <pm:border xmlns:pm="smNativeData" id="1777560623">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -724,7 +713,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
+          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
         </ext>
       </extLst>
     </border>
@@ -743,7 +732,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
+          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
         </ext>
       </extLst>
     </border>
@@ -762,7 +751,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
+          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
         </ext>
       </extLst>
     </border>
@@ -781,26 +770,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777486352"/>
+          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
         </ext>
       </extLst>
     </border>
@@ -813,7 +783,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -847,6 +817,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -862,7 +835,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -875,7 +848,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -886,7 +859,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -899,7 +872,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -910,7 +883,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -923,7 +896,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -934,7 +907,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -947,7 +920,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -958,7 +931,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -971,7 +944,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -982,7 +955,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -995,7 +968,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1006,7 +979,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1019,7 +992,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1030,7 +1003,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1043,7 +1016,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1054,7 +1027,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1067,7 +1040,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1078,7 +1051,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1091,7 +1064,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1102,7 +1075,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1115,7 +1088,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1126,7 +1099,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1139,7 +1112,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1150,7 +1123,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1163,7 +1136,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1174,7 +1147,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1187,7 +1160,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1198,7 +1171,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1211,7 +1184,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1222,7 +1195,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1235,7 +1208,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1246,7 +1219,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1259,7 +1232,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1270,7 +1243,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1283,7 +1256,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1294,7 +1267,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1307,7 +1280,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1318,7 +1291,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1331,7 +1304,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1342,7 +1315,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1355,7 +1328,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1366,7 +1339,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1379,7 +1352,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1390,7 +1363,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1403,7 +1376,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1414,7 +1387,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1427,7 +1400,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1438,7 +1411,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1451,7 +1424,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1462,7 +1435,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1475,7 +1448,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1486,7 +1459,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1499,7 +1472,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1510,7 +1483,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1523,7 +1496,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1534,7 +1507,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1547,7 +1520,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1558,7 +1531,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1571,7 +1544,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1582,7 +1555,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777486352" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1595,7 +1568,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777486352" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1605,10 +1578,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1777486352" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1777560623" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1777486352" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1777560623" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3038,7 +3011,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3047,14 +3020,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3113,7 +3086,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3124,14 +3097,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3182,7 +3155,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3193,14 +3166,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3289,7 +3262,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3300,14 +3273,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3360,7 +3333,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3371,14 +3344,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3462,7 +3435,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3473,14 +3446,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3571,7 +3544,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3582,14 +3555,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3628,7 +3601,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3639,14 +3612,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3785,17 +3758,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:4">
       <c r="A17" s="9" t="s">
         <v>65</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>28</v>
@@ -3804,68 +3780,68 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -3876,7 +3852,7 @@
         <v>26</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -3887,7 +3863,7 @@
         <v>26</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -3898,7 +3874,7 @@
         <v>26</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -3916,7 +3892,7 @@
         <v>26</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -3927,7 +3903,7 @@
         <v>26</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -3961,7 +3937,7 @@
         <v>26</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4002,7 +3978,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4013,14 +3989,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4091,7 +4067,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4102,14 +4078,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4169,7 +4145,7 @@
     </row>
     <row r="8" spans="2:2">
       <c r="B8" s="13" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4190,7 +4166,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4201,14 +4177,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4320,7 +4296,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4331,14 +4307,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4403,7 +4379,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777486352" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4414,14 +4390,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777486352" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777486352" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added remaining tests for TypedArray (#913)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="4" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="592"/>
+    <workbookView activeTab="13" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="592"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -21,21 +21,22 @@
     <sheet name="Stream handling" sheetId="11" r:id="rId14"/>
     <sheet name="Metadata" sheetId="12" r:id="rId15"/>
     <sheet name="Options" sheetId="13" r:id="rId16"/>
+    <sheet name="JS-compat objects" sheetId="14" r:id="rId17"/>
   </sheets>
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1777560623" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1777560623" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1777560623" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1777560623"/>
+      <pm:revision xmlns:pm="smNativeData" day="1777923981" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1777923981" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1777923981" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1777923981"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="135">
   <si>
     <t>Context</t>
   </si>
@@ -404,6 +405,42 @@
   </si>
   <si>
     <t>Disabling IO redirection</t>
+  </si>
+  <si>
+    <t>ArrayBuffer</t>
+  </si>
+  <si>
+    <t>Int8Array</t>
+  </si>
+  <si>
+    <t>Int16Array</t>
+  </si>
+  <si>
+    <t>Int32Array</t>
+  </si>
+  <si>
+    <t>Int64Array</t>
+  </si>
+  <si>
+    <t>Uint8Array</t>
+  </si>
+  <si>
+    <t>Uint16Array</t>
+  </si>
+  <si>
+    <t>Uint32Array</t>
+  </si>
+  <si>
+    <t>Uint64Array</t>
+  </si>
+  <si>
+    <t>Float16Array</t>
+  </si>
+  <si>
+    <t>Float32Array</t>
+  </si>
+  <si>
+    <t>Float64Array</t>
   </si>
 </sst>
 </file>
@@ -433,7 +470,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -448,7 +485,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -463,7 +500,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -479,7 +516,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777560623" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -501,7 +538,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -512,7 +549,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -523,7 +560,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -534,7 +571,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -545,7 +582,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -556,7 +593,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -567,18 +604,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFB3B3"/>
+        <fgColor rgb="FFFFC000"/>
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -600,7 +637,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
+          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
         </ext>
       </extLst>
     </border>
@@ -619,7 +656,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623">
+          <pm:border xmlns:pm="smNativeData" id="1777923981">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -641,7 +678,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623">
+          <pm:border xmlns:pm="smNativeData" id="1777923981">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -665,7 +702,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623">
+          <pm:border xmlns:pm="smNativeData" id="1777923981">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -689,7 +726,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623">
+          <pm:border xmlns:pm="smNativeData" id="1777923981">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -713,7 +750,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
+          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
         </ext>
       </extLst>
     </border>
@@ -732,7 +769,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
+          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
         </ext>
       </extLst>
     </border>
@@ -751,7 +788,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
+          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
         </ext>
       </extLst>
     </border>
@@ -770,7 +807,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777560623"/>
+          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
         </ext>
       </extLst>
     </border>
@@ -783,7 +820,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -817,9 +854,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -835,7 +869,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -848,7 +882,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -859,7 +893,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -872,7 +906,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -883,7 +917,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -896,7 +930,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -907,7 +941,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -920,7 +954,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -931,7 +965,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -944,7 +978,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -955,7 +989,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -968,7 +1002,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -979,7 +1013,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -992,7 +1026,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1003,7 +1037,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1016,7 +1050,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1027,7 +1061,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1040,7 +1074,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1051,7 +1085,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1064,7 +1098,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1075,7 +1109,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1088,7 +1122,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1099,7 +1133,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1112,7 +1146,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1123,7 +1157,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1136,7 +1170,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1147,7 +1181,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1160,7 +1194,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1171,7 +1205,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1184,7 +1218,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1195,7 +1229,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1208,7 +1242,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1219,7 +1253,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1232,7 +1266,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1243,7 +1277,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1256,7 +1290,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1267,7 +1301,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1280,7 +1314,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1291,7 +1325,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1304,7 +1338,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1315,7 +1349,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1328,7 +1362,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1339,7 +1373,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1352,7 +1386,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1363,7 +1397,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1376,7 +1410,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1387,7 +1421,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1400,7 +1434,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1411,7 +1445,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1424,7 +1458,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1435,7 +1469,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1448,7 +1482,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1459,7 +1493,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1472,7 +1506,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1483,7 +1517,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1496,7 +1530,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1507,7 +1541,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1520,7 +1554,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1531,7 +1565,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1544,7 +1578,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1555,7 +1589,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777560623" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1568,7 +1602,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777560623" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1578,10 +1612,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1777560623" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1777923981" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1777560623" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1777923981" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3011,7 +3045,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3020,14 +3054,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3086,7 +3120,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3097,14 +3131,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3155,7 +3189,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3166,14 +3200,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3262,7 +3296,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3273,14 +3307,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3333,7 +3367,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3344,14 +3378,162 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+        <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+        <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+      </pm:sheetPrefs>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="9" defaultColWidth="10.000000" defaultRowHeight="15.40"/>
+  <cols>
+    <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
+    <col min="2" max="16384" width="8.669643" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="12"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="6"/>
+      <c r="B2" s="12"/>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+  </mergeCells>
+  <printOptions>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+      </ext>
+    </extLst>
+  </printOptions>
+  <pageMargins left="1.000000" right="1.000000" top="1.000000" bottom="1.000000" header="0.393750" footer="0.393750"/>
+  <pageSetup paperSize="1" fitToWidth="0" fitToHeight="1" pageOrder="overThenDown"/>
+  <headerFooter>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+      </ext>
+    </extLst>
+  </headerFooter>
+  <extLst>
+    <ext uri="smNativeData">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3435,7 +3617,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3446,14 +3628,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3544,7 +3726,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3555,14 +3737,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3601,7 +3783,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3612,14 +3794,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3765,7 +3947,7 @@
       <c r="B17" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="13" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3774,9 +3956,11 @@
         <v>67</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="9" t="s">
@@ -3978,7 +4162,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3989,14 +4173,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4067,7 +4251,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4078,14 +4262,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4166,7 +4350,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4177,14 +4361,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4296,7 +4480,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4307,14 +4491,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4379,7 +4563,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777560623" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4390,14 +4574,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777560623" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777560623" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added remaining fcall test cases (#908)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="13" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="592"/>
+    <workbookView activeTab="4" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="592"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1777923981" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1777923981" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1777923981" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1777923981"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778016998" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778016998" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778016998" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778016998"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="135">
   <si>
     <t>Context</t>
   </si>
@@ -470,7 +470,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -485,7 +485,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -500,7 +500,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -516,7 +516,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777923981" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -525,7 +525,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,7 +538,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -549,7 +549,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -560,7 +560,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -571,7 +571,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -582,7 +582,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -593,7 +593,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -604,24 +604,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -637,7 +626,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
+          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
         </ext>
       </extLst>
     </border>
@@ -656,7 +645,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981">
+          <pm:border xmlns:pm="smNativeData" id="1778016998">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -678,7 +667,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981">
+          <pm:border xmlns:pm="smNativeData" id="1778016998">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -702,7 +691,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981">
+          <pm:border xmlns:pm="smNativeData" id="1778016998">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -726,7 +715,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981">
+          <pm:border xmlns:pm="smNativeData" id="1778016998">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -750,7 +739,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
+          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
         </ext>
       </extLst>
     </border>
@@ -769,7 +758,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
+          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
         </ext>
       </extLst>
     </border>
@@ -788,26 +777,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777923981"/>
+          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
         </ext>
       </extLst>
     </border>
@@ -869,7 +839,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -882,7 +852,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -893,7 +863,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -906,7 +876,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -917,7 +887,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -930,7 +900,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -941,7 +911,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -954,7 +924,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -965,7 +935,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -978,7 +948,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -989,7 +959,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1002,7 +972,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1013,7 +983,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1026,7 +996,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1037,7 +1007,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1050,7 +1020,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1061,7 +1031,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1074,7 +1044,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1085,7 +1055,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1098,7 +1068,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1109,7 +1079,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1122,7 +1092,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1133,7 +1103,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1146,7 +1116,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1157,7 +1127,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1170,7 +1140,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1181,7 +1151,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1194,7 +1164,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1205,7 +1175,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1218,7 +1188,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1229,7 +1199,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1242,7 +1212,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1253,7 +1223,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1266,7 +1236,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1277,7 +1247,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1290,7 +1260,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1301,7 +1271,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1314,7 +1284,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1325,7 +1295,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1338,7 +1308,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1349,7 +1319,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1362,7 +1332,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1373,7 +1343,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1386,7 +1356,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1397,7 +1367,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1410,7 +1380,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1421,7 +1391,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1434,7 +1404,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1445,7 +1415,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1458,7 +1428,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1469,7 +1439,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1482,7 +1452,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1493,7 +1463,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1506,7 +1476,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1517,7 +1487,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1530,7 +1500,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1541,7 +1511,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1554,7 +1524,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1565,7 +1535,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1578,7 +1548,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1589,7 +1559,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1777923981" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1602,7 +1572,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1777923981" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1612,10 +1582,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1777923981" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778016998" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1777923981" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778016998" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3045,7 +3015,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3054,14 +3024,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3120,7 +3090,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3131,14 +3101,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3189,7 +3159,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3200,14 +3170,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3296,7 +3266,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3307,14 +3277,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3367,7 +3337,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3378,14 +3348,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3517,7 +3487,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3526,14 +3496,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3617,7 +3587,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3628,14 +3598,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3726,7 +3696,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3737,14 +3707,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3783,7 +3753,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3794,14 +3764,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4065,8 +4035,12 @@
       <c r="A28" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B28" s="10"/>
-      <c r="D28" s="10"/>
+      <c r="B28" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
@@ -4094,15 +4068,23 @@
       <c r="A31" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B31" s="10"/>
-      <c r="D31" s="10"/>
+      <c r="B31" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B32" s="10"/>
-      <c r="D32" s="10"/>
+      <c r="B32" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="9" t="s">
@@ -4162,7 +4144,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4173,14 +4155,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4251,7 +4233,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4262,14 +4244,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4350,7 +4332,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4361,14 +4343,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4480,7 +4462,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4491,14 +4473,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4563,7 +4545,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777923981" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4574,14 +4556,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777923981" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777923981" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Fixed memory leaks (#908)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778016998" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778016998" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778016998" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778016998"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778024125" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778024125" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778024125" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778024125"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="134">
   <si>
     <t>Context</t>
   </si>
@@ -236,16 +236,13 @@
     <t>Handle recursive structure</t>
   </si>
   <si>
+    <t>Return const pointer</t>
+  </si>
+  <si>
     <t>leak</t>
   </si>
   <si>
-    <t>Return const pointer</t>
-  </si>
-  <si>
     <t>Accept multiple pointers</t>
-  </si>
-  <si>
-    <t>segfault</t>
   </si>
   <si>
     <t>Accept C pointers</t>
@@ -470,7 +467,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -485,7 +482,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -500,7 +497,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -516,7 +513,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778016998" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -525,7 +522,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,7 +535,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -549,7 +546,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -560,7 +557,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -571,7 +568,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -582,7 +579,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -593,24 +590,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -626,7 +612,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
+          <pm:border xmlns:pm="smNativeData" id="1778024125"/>
         </ext>
       </extLst>
     </border>
@@ -645,7 +631,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998">
+          <pm:border xmlns:pm="smNativeData" id="1778024125">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -667,7 +653,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998">
+          <pm:border xmlns:pm="smNativeData" id="1778024125">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -691,7 +677,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998">
+          <pm:border xmlns:pm="smNativeData" id="1778024125">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -715,7 +701,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998">
+          <pm:border xmlns:pm="smNativeData" id="1778024125">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -739,7 +725,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
+          <pm:border xmlns:pm="smNativeData" id="1778024125"/>
         </ext>
       </extLst>
     </border>
@@ -758,26 +744,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778016998"/>
+          <pm:border xmlns:pm="smNativeData" id="1778024125"/>
         </ext>
       </extLst>
     </border>
@@ -839,7 +806,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -852,7 +819,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -863,7 +830,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -876,7 +843,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -887,7 +854,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -900,7 +867,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -911,7 +878,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -924,7 +891,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -935,7 +902,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -948,7 +915,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -959,7 +926,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -972,7 +939,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -983,7 +950,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -996,7 +963,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1007,7 +974,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1020,7 +987,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1031,7 +998,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1044,7 +1011,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1055,7 +1022,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1068,7 +1035,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1079,7 +1046,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1092,7 +1059,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1103,7 +1070,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1116,7 +1083,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1127,7 +1094,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1140,7 +1107,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1151,7 +1118,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1164,7 +1131,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1175,7 +1142,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1188,7 +1155,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1199,7 +1166,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1212,7 +1179,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1223,7 +1190,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1236,7 +1203,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1247,7 +1214,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1260,7 +1227,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1271,7 +1238,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1284,7 +1251,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1295,7 +1262,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1308,7 +1275,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1319,7 +1286,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1332,7 +1299,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1343,7 +1310,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1356,7 +1323,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1367,7 +1334,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1380,7 +1347,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1391,7 +1358,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1404,7 +1371,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1415,7 +1382,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1428,7 +1395,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1439,7 +1406,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1452,7 +1419,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1463,7 +1430,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1476,7 +1443,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1487,7 +1454,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1500,7 +1467,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1511,7 +1478,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1524,7 +1491,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1535,7 +1502,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1548,7 +1515,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1559,7 +1526,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778016998" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1572,7 +1539,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778016998" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1582,10 +1549,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778016998" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778024125" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778016998" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778024125" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3015,7 +2982,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3024,14 +2991,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3060,25 +3027,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -3090,7 +3057,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3101,14 +3068,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3159,7 +3126,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3170,14 +3137,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3206,55 +3173,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3266,7 +3233,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3277,14 +3244,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3313,19 +3280,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3337,7 +3304,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3348,14 +3315,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3385,7 +3352,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3393,7 +3360,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3401,7 +3368,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3409,7 +3376,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -3417,7 +3384,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -3425,7 +3392,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -3433,7 +3400,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -3441,7 +3408,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -3449,7 +3416,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -3457,7 +3424,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -3465,7 +3432,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -3473,7 +3440,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -3487,7 +3454,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3496,14 +3463,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3587,7 +3554,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3598,14 +3565,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3696,7 +3663,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3707,14 +3674,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3753,7 +3720,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3764,14 +3731,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3917,19 +3884,17 @@
       <c r="B17" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>66</v>
-      </c>
+      <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>67</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -3939,156 +3904,128 @@
       <c r="B19" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>69</v>
-      </c>
+      <c r="D19" s="10"/>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>69</v>
-      </c>
+      <c r="D20" s="10"/>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>69</v>
-      </c>
+      <c r="D21" s="10"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="10" t="s">
-        <v>69</v>
-      </c>
+      <c r="D22" s="10"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="10" t="s">
-        <v>69</v>
-      </c>
+      <c r="D23" s="10"/>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D24" s="10"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D25" s="10"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D26" s="10"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D27" s="10"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="10" t="s">
-        <v>69</v>
-      </c>
+      <c r="D28" s="10"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D29" s="10"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D30" s="10"/>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D31" s="10"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D32" s="10"/>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>28</v>
@@ -4097,14 +4034,12 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="D34" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4144,7 +4079,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4155,14 +4090,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4191,31 +4126,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -4233,7 +4168,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4244,14 +4179,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4280,7 +4215,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4288,7 +4223,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4296,7 +4231,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4305,13 +4240,13 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="8" spans="2:2">
       <c r="B8" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -4332,7 +4267,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4343,14 +4278,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4379,7 +4314,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>28</v>
@@ -4387,13 +4322,13 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4401,7 +4336,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>28</v>
@@ -4409,7 +4344,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4417,20 +4352,20 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -4462,7 +4397,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4473,14 +4408,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4509,31 +4444,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -4545,7 +4480,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778016998" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4556,14 +4491,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778016998" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778016998" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Implemented proper disposal of callback thunk (#908)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="4" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="592"/>
+    <workbookView activeTab="4" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778024125" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778024125" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778024125" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778024125"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778071100" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778071100" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778071100" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778071100"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="134">
   <si>
     <t>Context</t>
   </si>
@@ -239,82 +239,82 @@
     <t>Return const pointer</t>
   </si>
   <si>
+    <t>Accept multiple pointers</t>
+  </si>
+  <si>
+    <t>Accept C pointers</t>
+  </si>
+  <si>
+    <t>Return multiple pointers</t>
+  </si>
+  <si>
+    <t>Return C pointers</t>
+  </si>
+  <si>
+    <t>Modify a pointer target</t>
+  </si>
+  <si>
+    <t>Call C functions</t>
+  </si>
+  <si>
+    <t>Call variadic functions</t>
+  </si>
+  <si>
+    <t>Pass unsigned in to variadic function</t>
+  </si>
+  <si>
+    <t>Write to file using fwrite</t>
+  </si>
+  <si>
+    <t>Read from file using fread</t>
+  </si>
+  <si>
+    <t>Call printf</t>
+  </si>
+  <si>
+    <t>Call fprintf</t>
+  </si>
+  <si>
+    <t>Call sprintf</t>
+  </si>
+  <si>
+    <t>Call snprintf</t>
+  </si>
+  <si>
+    <t>Handle immediate promise fulfillment</t>
+  </si>
+  <si>
+    <t>Apply transform to return value</t>
+  </si>
+  <si>
+    <t>Free function thunk</t>
+  </si>
+  <si>
+    <t>Floatng point args</t>
+  </si>
+  <si>
+    <t>Struct args</t>
+  </si>
+  <si>
+    <t>Array args</t>
+  </si>
+  <si>
+    <t>Slice args</t>
+  </si>
+  <si>
+    <t>Create internal slice</t>
+  </si>
+  <si>
+    <t>Allocate memory for string</t>
+  </si>
+  <si>
+    <t>Retain allocator</t>
+  </si>
+  <si>
+    <t>Return allocator</t>
+  </si>
+  <si>
     <t>leak</t>
-  </si>
-  <si>
-    <t>Accept multiple pointers</t>
-  </si>
-  <si>
-    <t>Accept C pointers</t>
-  </si>
-  <si>
-    <t>Return multiple pointers</t>
-  </si>
-  <si>
-    <t>Return C pointers</t>
-  </si>
-  <si>
-    <t>Modify a pointer target</t>
-  </si>
-  <si>
-    <t>Call C functions</t>
-  </si>
-  <si>
-    <t>Call variadic functions</t>
-  </si>
-  <si>
-    <t>Pass unsigned in to variadic function</t>
-  </si>
-  <si>
-    <t>Write to file using fwrite</t>
-  </si>
-  <si>
-    <t>Read from file using fread</t>
-  </si>
-  <si>
-    <t>Call printf</t>
-  </si>
-  <si>
-    <t>Call fprintf</t>
-  </si>
-  <si>
-    <t>Call sprintf</t>
-  </si>
-  <si>
-    <t>Call snprintf</t>
-  </si>
-  <si>
-    <t>Handle immediate promise fulfillment</t>
-  </si>
-  <si>
-    <t>Apply transform to return value</t>
-  </si>
-  <si>
-    <t>Free function thunk</t>
-  </si>
-  <si>
-    <t>Floatng point args</t>
-  </si>
-  <si>
-    <t>Struct args</t>
-  </si>
-  <si>
-    <t>Array args</t>
-  </si>
-  <si>
-    <t>Slice args</t>
-  </si>
-  <si>
-    <t>Create internal slice</t>
-  </si>
-  <si>
-    <t>Allocate memory for string</t>
-  </si>
-  <si>
-    <t>Retain allocator</t>
-  </si>
-  <si>
-    <t>Return allocator</t>
   </si>
   <si>
     <t>Thread creation</t>
@@ -467,7 +467,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -482,7 +482,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -497,7 +497,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -513,7 +513,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778024125" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -522,7 +522,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,7 +535,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -546,7 +546,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -557,7 +557,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -568,7 +568,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -579,7 +579,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -590,13 +590,35 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -612,7 +634,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778024125"/>
+          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
         </ext>
       </extLst>
     </border>
@@ -631,7 +653,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778024125">
+          <pm:border xmlns:pm="smNativeData" id="1778071100">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -653,7 +675,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778024125">
+          <pm:border xmlns:pm="smNativeData" id="1778071100">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -677,7 +699,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778024125">
+          <pm:border xmlns:pm="smNativeData" id="1778071100">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -701,7 +723,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778024125">
+          <pm:border xmlns:pm="smNativeData" id="1778071100">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -725,7 +747,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778024125"/>
+          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
         </ext>
       </extLst>
     </border>
@@ -744,7 +766,45 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778024125"/>
+          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
         </ext>
       </extLst>
     </border>
@@ -806,7 +866,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -819,7 +879,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -830,7 +890,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -843,7 +903,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -854,7 +914,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -867,7 +927,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -878,7 +938,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -891,7 +951,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -902,7 +962,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -915,7 +975,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -926,7 +986,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -939,7 +999,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -950,7 +1010,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -963,7 +1023,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -974,7 +1034,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -987,7 +1047,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -998,7 +1058,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1011,7 +1071,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1022,7 +1082,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1035,7 +1095,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1046,7 +1106,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1059,7 +1119,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1070,7 +1130,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1083,7 +1143,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1094,7 +1154,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1107,7 +1167,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1118,7 +1178,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1131,7 +1191,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1142,7 +1202,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1155,7 +1215,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1166,7 +1226,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1179,7 +1239,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1190,7 +1250,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1203,7 +1263,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1214,7 +1274,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1227,7 +1287,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1238,7 +1298,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1251,7 +1311,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1262,7 +1322,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1275,7 +1335,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1286,7 +1346,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1299,7 +1359,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1310,7 +1370,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1323,7 +1383,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1334,7 +1394,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1347,7 +1407,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1358,7 +1418,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1371,7 +1431,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1382,7 +1442,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1395,7 +1455,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1406,7 +1466,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1419,7 +1479,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1430,7 +1490,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1443,7 +1503,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1454,7 +1514,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1467,7 +1527,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1478,7 +1538,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1491,7 +1551,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1502,7 +1562,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1515,7 +1575,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1526,7 +1586,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778024125" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1539,7 +1599,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778024125" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1549,10 +1609,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778024125" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778071100" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778024125" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778071100" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -2982,7 +3042,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2991,14 +3051,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3057,7 +3117,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3068,14 +3128,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3126,7 +3186,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3137,14 +3197,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3233,7 +3293,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3244,14 +3304,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3304,7 +3364,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3315,14 +3375,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3454,7 +3514,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3463,14 +3523,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3554,7 +3614,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3565,14 +3625,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3663,7 +3723,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3674,14 +3734,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3720,7 +3780,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3731,14 +3791,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3893,13 +3953,11 @@
       <c r="B18" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="10" t="s">
-        <v>67</v>
-      </c>
+      <c r="D18" s="10"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>26</v>
@@ -3908,7 +3966,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>26</v>
@@ -3917,7 +3975,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>26</v>
@@ -3926,7 +3984,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
@@ -3935,7 +3993,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
@@ -3944,7 +4002,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>26</v>
@@ -3953,7 +4011,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>26</v>
@@ -3962,7 +4020,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>26</v>
@@ -3971,7 +4029,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>26</v>
@@ -3980,7 +4038,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>26</v>
@@ -3989,7 +4047,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>26</v>
@@ -3998,7 +4056,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>26</v>
@@ -4007,7 +4065,7 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>26</v>
@@ -4016,7 +4074,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>26</v>
@@ -4025,16 +4083,16 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D33" s="10"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>26</v>
@@ -4079,7 +4137,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4090,14 +4148,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4126,31 +4184,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -4168,7 +4226,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4179,14 +4237,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4215,7 +4273,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4223,7 +4281,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4231,7 +4289,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4240,13 +4298,13 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="8" spans="2:2">
       <c r="B8" s="13" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -4267,7 +4325,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4278,14 +4336,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4397,7 +4455,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4408,14 +4466,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4480,7 +4538,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778024125" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4491,14 +4549,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778024125" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778024125" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added tests for iterator (#917)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="4" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
+    <workbookView activeTab="9" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778071100" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778071100" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778071100" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778071100"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778091295" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778091295" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778091295" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778091295"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="135">
   <si>
     <t>Context</t>
   </si>
@@ -356,13 +356,16 @@
     <t>Using zig-duckdb</t>
   </si>
   <si>
+    <t>Struct iterator</t>
+  </si>
+  <si>
+    <t>Union iterator</t>
+  </si>
+  <si>
+    <t>Opaque iterator</t>
+  </si>
+  <si>
     <t>std.mem.SplitIterator</t>
-  </si>
-  <si>
-    <t>std.zip.Iterator</t>
-  </si>
-  <si>
-    <t>std.fs.Dir.Iterator</t>
   </si>
   <si>
     <t>std.fs.path.ComponentIterator</t>
@@ -467,7 +470,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778091295" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -482,7 +485,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778091295" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -497,7 +500,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778091295" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -513,7 +516,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778071100" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778091295" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -522,7 +525,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,7 +538,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -546,7 +549,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -557,7 +560,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -568,7 +571,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -579,7 +582,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -590,7 +593,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -601,24 +604,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFB3B3"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -634,7 +626,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
+          <pm:border xmlns:pm="smNativeData" id="1778091295"/>
         </ext>
       </extLst>
     </border>
@@ -653,7 +645,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100">
+          <pm:border xmlns:pm="smNativeData" id="1778091295">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -675,7 +667,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100">
+          <pm:border xmlns:pm="smNativeData" id="1778091295">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -699,7 +691,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100">
+          <pm:border xmlns:pm="smNativeData" id="1778091295">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -723,7 +715,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100">
+          <pm:border xmlns:pm="smNativeData" id="1778091295">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -747,7 +739,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
+          <pm:border xmlns:pm="smNativeData" id="1778091295"/>
         </ext>
       </extLst>
     </border>
@@ -766,7 +758,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
+          <pm:border xmlns:pm="smNativeData" id="1778091295"/>
         </ext>
       </extLst>
     </border>
@@ -785,26 +777,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778071100"/>
+          <pm:border xmlns:pm="smNativeData" id="1778091295"/>
         </ext>
       </extLst>
     </border>
@@ -817,7 +790,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -851,6 +824,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -866,7 +842,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -879,7 +855,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -890,7 +866,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -903,7 +879,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -914,7 +890,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -927,7 +903,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -938,7 +914,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -951,7 +927,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -962,7 +938,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -975,7 +951,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -986,7 +962,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -999,7 +975,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1010,7 +986,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1023,7 +999,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1034,7 +1010,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1047,7 +1023,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1058,7 +1034,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1071,7 +1047,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1082,7 +1058,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1095,7 +1071,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1106,7 +1082,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1119,7 +1095,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1130,7 +1106,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1143,7 +1119,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1154,7 +1130,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1167,7 +1143,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1178,7 +1154,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1191,7 +1167,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1202,7 +1178,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1215,7 +1191,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1226,7 +1202,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1239,7 +1215,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1250,7 +1226,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1263,7 +1239,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1274,7 +1250,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1287,7 +1263,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1298,7 +1274,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1311,7 +1287,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1322,7 +1298,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1335,7 +1311,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1346,7 +1322,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1359,7 +1335,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1370,7 +1346,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1383,7 +1359,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1394,7 +1370,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1407,7 +1383,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1418,7 +1394,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1431,7 +1407,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1442,7 +1418,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1455,7 +1431,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1466,7 +1442,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1479,7 +1455,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1490,7 +1466,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1503,7 +1479,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1514,7 +1490,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1527,7 +1503,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1538,7 +1514,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1551,7 +1527,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1562,7 +1538,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1575,7 +1551,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1586,7 +1562,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778071100" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778091295" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1599,7 +1575,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778071100" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778091295" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1609,10 +1585,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778071100" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778091295" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778071100" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778091295" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3042,7 +3018,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3051,14 +3027,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3069,7 +3045,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
@@ -3085,29 +3061,56 @@
       <c r="A2" s="6"/>
       <c r="B2" s="12"/>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="10"/>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B4" s="10"/>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="15"/>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="B5" s="10"/>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="15"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>92</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3117,7 +3120,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3128,14 +3131,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3186,7 +3189,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3197,14 +3200,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3233,55 +3236,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3293,7 +3296,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3304,14 +3307,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3340,19 +3343,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3364,7 +3367,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3375,14 +3378,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3412,7 +3415,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3420,7 +3423,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3428,7 +3431,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3436,7 +3439,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -3444,7 +3447,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -3452,7 +3455,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -3460,7 +3463,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -3468,7 +3471,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -3476,7 +3479,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -3484,7 +3487,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -3492,7 +3495,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -3500,7 +3503,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -3514,7 +3517,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3523,14 +3526,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3614,7 +3617,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3625,14 +3628,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3723,7 +3726,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3734,14 +3737,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3780,7 +3783,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3791,14 +3794,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4137,7 +4140,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4148,14 +4151,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4226,7 +4229,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4237,14 +4240,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4325,7 +4328,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4336,14 +4339,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4455,7 +4458,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4466,14 +4469,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4538,7 +4541,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778071100" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778091295" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4549,14 +4552,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778071100" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778091295" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778071100" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778091295" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added tests related to stream handling (#918)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="9" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
+    <workbookView activeTab="10" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778094077" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778094077" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778094077" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778094077"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778105145" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778105145" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778105145" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778105145"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="159">
   <si>
     <t>Context</t>
   </si>
@@ -369,6 +369,78 @@
   </si>
   <si>
     <t>std.fs.path.ComponentIterator</t>
+  </si>
+  <si>
+    <t>Read from file</t>
+  </si>
+  <si>
+    <t>Read from file in main thread</t>
+  </si>
+  <si>
+    <t>Open and read file in main thread</t>
+  </si>
+  <si>
+    <t>Fallback to file system</t>
+  </si>
+  <si>
+    <t>Open file through FS using posix functions</t>
+  </si>
+  <si>
+    <t>Open file through FS using libc functions</t>
+  </si>
+  <si>
+    <t>Open file through direct syscall</t>
+  </si>
+  <si>
+    <t>Open and read file using posix functions</t>
+  </si>
+  <si>
+    <t>Open and read file using libc functions</t>
+  </si>
+  <si>
+    <t>Seek to particular position</t>
+  </si>
+  <si>
+    <t>Seek to particular position in thread</t>
+  </si>
+  <si>
+    <t>Open file and seek to particular position using posix functions</t>
+  </si>
+  <si>
+    <t>Open file and seek to particular position using libc functions</t>
+  </si>
+  <si>
+    <t>Open file and seek to particular position using win32 functions</t>
+  </si>
+  <si>
+    <t>Open file through FS using win32 function</t>
+  </si>
+  <si>
+    <t>Obtain expected position after seek using posix function</t>
+  </si>
+  <si>
+    <t>Obtain expected position after seek using libc function</t>
+  </si>
+  <si>
+    <t>Save and restore file position using libc functions</t>
+  </si>
+  <si>
+    <t>Write to file</t>
+  </si>
+  <si>
+    <t>Write to file in main thread</t>
+  </si>
+  <si>
+    <t>Open and write to file in main thread</t>
+  </si>
+  <si>
+    <t>Open and write to file using posix functions</t>
+  </si>
+  <si>
+    <t>Open and write to file using libc functions</t>
+  </si>
+  <si>
+    <t>Open and write to file using win32 functions</t>
   </si>
   <si>
     <t>Field as string</t>
@@ -470,7 +542,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778094077" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -485,7 +557,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778094077" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -500,7 +572,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778094077" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -516,7 +588,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778094077" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -525,7 +597,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,7 +610,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -549,7 +621,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -560,7 +632,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -571,7 +643,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -582,7 +654,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -593,7 +665,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -604,13 +676,24 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -626,7 +709,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077"/>
+          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
         </ext>
       </extLst>
     </border>
@@ -645,7 +728,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077">
+          <pm:border xmlns:pm="smNativeData" id="1778105145">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -667,7 +750,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077">
+          <pm:border xmlns:pm="smNativeData" id="1778105145">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -691,7 +774,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077">
+          <pm:border xmlns:pm="smNativeData" id="1778105145">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -715,7 +798,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077">
+          <pm:border xmlns:pm="smNativeData" id="1778105145">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -739,7 +822,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077"/>
+          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
         </ext>
       </extLst>
     </border>
@@ -758,7 +841,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077"/>
+          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
         </ext>
       </extLst>
     </border>
@@ -777,7 +860,26 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778094077"/>
+          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
         </ext>
       </extLst>
     </border>
@@ -833,13 +935,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="31">
+  <dxfs count="37">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -852,7 +954,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -863,7 +965,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -876,7 +978,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -887,7 +989,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -900,7 +1002,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -911,7 +1013,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -924,7 +1026,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -935,7 +1037,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -948,7 +1050,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -959,7 +1061,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -972,7 +1074,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -983,7 +1085,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -996,7 +1098,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1007,7 +1109,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1020,7 +1122,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1031,7 +1133,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1044,7 +1146,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1055,7 +1157,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1068,7 +1170,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1079,7 +1181,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1092,7 +1194,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1103,7 +1205,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1116,7 +1218,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1127,7 +1229,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1140,7 +1242,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1151,7 +1253,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1164,7 +1266,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1175,7 +1277,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1188,7 +1290,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1199,7 +1301,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1212,7 +1314,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1223,7 +1325,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1236,7 +1338,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1247,7 +1349,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1260,7 +1362,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1271,7 +1373,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1284,7 +1386,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1295,7 +1397,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1308,7 +1410,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1319,7 +1421,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1332,7 +1434,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1343,7 +1445,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1356,7 +1458,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1367,7 +1469,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1380,7 +1482,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1391,7 +1493,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1404,7 +1506,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1415,7 +1517,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1428,7 +1530,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1439,7 +1541,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1452,7 +1554,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1463,7 +1565,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1476,7 +1578,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1487,7 +1589,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1500,7 +1602,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1511,7 +1613,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1524,7 +1626,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1535,7 +1637,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1548,7 +1650,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1559,7 +1661,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778094077" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1572,7 +1674,151 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778094077" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1582,10 +1828,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778094077" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778105145" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778094077" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778105145" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3015,7 +3261,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3024,14 +3270,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3108,10 +3354,20 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B7">
+    <cfRule type="cellIs" dxfId="33" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B7">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3122,14 +3378,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3140,10 +3396,10 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
-    <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
+    <col min="1" max="1" width="55.482143" customWidth="1" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3157,30 +3413,196 @@
       <c r="B2" s="12"/>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="9"/>
+      <c r="A3" s="9" t="s">
+        <v>111</v>
+      </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="9"/>
+      <c r="A4" s="9" t="s">
+        <v>112</v>
+      </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
+      <c r="A6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B12" s="10"/>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="10"/>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B16" s="10"/>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B17" s="10"/>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B20" s="10"/>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="10"/>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="10"/>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B26">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B26">
+    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3191,14 +3613,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3227,55 +3649,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3287,7 +3709,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3298,14 +3720,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3334,19 +3756,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3358,7 +3780,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3369,14 +3791,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3406,7 +3828,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3414,7 +3836,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3422,7 +3844,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3430,7 +3852,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -3438,7 +3860,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -3446,7 +3868,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -3454,7 +3876,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -3462,7 +3884,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -3470,7 +3892,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -3478,7 +3900,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -3486,7 +3908,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -3494,7 +3916,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -3508,7 +3930,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3517,14 +3939,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3608,7 +4030,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3619,14 +4041,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3717,7 +4139,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3728,14 +4150,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3774,7 +4196,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3785,14 +4207,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4131,7 +4553,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4142,14 +4564,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4220,7 +4642,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4231,14 +4653,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4319,7 +4741,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4330,14 +4752,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4449,7 +4871,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4460,14 +4882,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4529,10 +4951,20 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B7">
+    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B7">
+    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778094077" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4543,14 +4975,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778094077" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778094077" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added more tests related to stream handling (#918)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778105145" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778105145" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778105145" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778105145"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778192348" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778192348" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778192348" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778192348"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="245">
   <si>
     <t>Context</t>
   </si>
@@ -441,6 +441,264 @@
   </si>
   <si>
     <t>Open and write to file using win32 functions</t>
+  </si>
+  <si>
+    <t>Obtain error code using libc function</t>
+  </si>
+  <si>
+    <t>Detect end of file using libc function</t>
+  </si>
+  <si>
+    <t>Rewind file using libc function</t>
+  </si>
+  <si>
+    <t>Check file access using posix function</t>
+  </si>
+  <si>
+    <t>Check access of file in directory using posix function</t>
+  </si>
+  <si>
+    <t>Check access of file in directory in file system using posix function</t>
+  </si>
+  <si>
+    <t>Open file in directory using posix function</t>
+  </si>
+  <si>
+    <t>Open file in directory in file system using posix function</t>
+  </si>
+  <si>
+    <t>Retrieve stat of file in directory using posix function</t>
+  </si>
+  <si>
+    <t>Retrieve stat of file in directory in file system using posix function</t>
+  </si>
+  <si>
+    <t>Decompress gzip file</t>
+  </si>
+  <si>
+    <t>Get stats of Uint8Array</t>
+  </si>
+  <si>
+    <t>Get stats of opened file using posix function</t>
+  </si>
+  <si>
+    <t>Get stats of opened file in file system using posix function</t>
+  </si>
+  <si>
+    <t>Get stats of file referenced by path using posix function</t>
+  </si>
+  <si>
+    <t>Get size of opened file using win32 function</t>
+  </si>
+  <si>
+    <t>Get stats of opened file using win32 function</t>
+  </si>
+  <si>
+    <t>Set access and last modified time of opened file using posix function</t>
+  </si>
+  <si>
+    <t>Set access and last modified time of opened file using futime</t>
+  </si>
+  <si>
+    <t>Set access and last modified time of file using posix function</t>
+  </si>
+  <si>
+    <t>Set access and last modified time of file using utime</t>
+  </si>
+  <si>
+    <t>Set access and last modified time of file in directory using posix function</t>
+  </si>
+  <si>
+    <t>Get directory entries</t>
+  </si>
+  <si>
+    <t>Get directory entries in thread</t>
+  </si>
+  <si>
+    <t>Perform sync operation using posix function</t>
+  </si>
+  <si>
+    <t>Perform datasync operation using posix function</t>
+  </si>
+  <si>
+    <t>Perform allocate operation using posix function</t>
+  </si>
+  <si>
+    <t>Open file in directory</t>
+  </si>
+  <si>
+    <t>Retrieve names of files in directory</t>
+  </si>
+  <si>
+    <t>Retrieve names of files in directory using posix functions</t>
+  </si>
+  <si>
+    <t>Create directory using posix function</t>
+  </si>
+  <si>
+    <t>Remove directory using posix function</t>
+  </si>
+  <si>
+    <t>Rename a file</t>
+  </si>
+  <si>
+    <t>Rename file in a directory</t>
+  </si>
+  <si>
+    <t>Rename file using posix function</t>
+  </si>
+  <si>
+    <t>Rename file in directory using posix function</t>
+  </si>
+  <si>
+    <t>Rename file in file system using posix function</t>
+  </si>
+  <si>
+    <t>Create symlink</t>
+  </si>
+  <si>
+    <t>Create symlink in directory</t>
+  </si>
+  <si>
+    <t>Create symlink using posix function</t>
+  </si>
+  <si>
+    <t>Create symlink in directory using posix function</t>
+  </si>
+  <si>
+    <t>Create symlink in file system using posix function</t>
+  </si>
+  <si>
+    <t>Create symlink using win32 function</t>
+  </si>
+  <si>
+    <t>Open and read from file using pread</t>
+  </si>
+  <si>
+    <t>Open and read from file using preadv</t>
+  </si>
+  <si>
+    <t>Open and read from file using readv</t>
+  </si>
+  <si>
+    <t>Open and write to file using pwrite</t>
+  </si>
+  <si>
+    <t>Open and write to file using pwritev</t>
+  </si>
+  <si>
+    <t>Open and write to file using writev</t>
+  </si>
+  <si>
+    <t>Set lock on file</t>
+  </si>
+  <si>
+    <t>Get lock on file using fcntl</t>
+  </si>
+  <si>
+    <t>Set lock on file using posix function</t>
+  </si>
+  <si>
+    <t>Set lock on file inside thread</t>
+  </si>
+  <si>
+    <t>Read lines from file using fgets</t>
+  </si>
+  <si>
+    <t>Read lines from stdin using fgets</t>
+  </si>
+  <si>
+    <t>Scan variables from a file using fscanf</t>
+  </si>
+  <si>
+    <t>Scan variables from stdin using scanf</t>
+  </si>
+  <si>
+    <t>Scan variables from web stream using scanf</t>
+  </si>
+  <si>
+    <t>Get characters from a file using fgetc</t>
+  </si>
+  <si>
+    <t>Get characters from stdin using getchar</t>
+  </si>
+  <si>
+    <t>Push character into stdin using ungetc</t>
+  </si>
+  <si>
+    <t>Flush open file using fflush</t>
+  </si>
+  <si>
+    <t>Delete file using win32 function</t>
+  </si>
+  <si>
+    <t>Delete file in directory</t>
+  </si>
+  <si>
+    <t>Remove directory using win32 function</t>
+  </si>
+  <si>
+    <t>Remove directory in directory</t>
+  </si>
+  <si>
+    <t>Make directory using win32 function</t>
+  </si>
+  <si>
+    <t>Make directory in directory</t>
+  </si>
+  <si>
+    <t>Read files using poll function</t>
+  </si>
+  <si>
+    <t>Redirect io from dynamically linked library</t>
+  </si>
+  <si>
+    <t>Create directory in file system using posix function</t>
+  </si>
+  <si>
+    <t>Create directory in another directory in file system using posix function</t>
+  </si>
+  <si>
+    <t>Remove directory in file system using posix function</t>
+  </si>
+  <si>
+    <t>Remove file in file system using posix function</t>
+  </si>
+  <si>
+    <t>Scan directory in file system using posix function</t>
+  </si>
+  <si>
+    <t>Read link using posix function</t>
+  </si>
+  <si>
+    <t>Fail to convert to file when useRedirection is false</t>
+  </si>
+  <si>
+    <t>Fail to convert to dir when useRedirection is false</t>
+  </si>
+  <si>
+    <t>Handle threads when useRedirection is false</t>
+  </si>
+  <si>
+    <t>Ignore offset to WriteFile when stream is unseekable</t>
+  </si>
+  <si>
+    <t>Copy read file to virtual file</t>
+  </si>
+  <si>
+    <t>Copy virtual file to virtual file</t>
+  </si>
+  <si>
+    <t>Copy virtual file to real file</t>
+  </si>
+  <si>
+    <t>Copy real file to virtual file using sendfile</t>
+  </si>
+  <si>
+    <t>Copy virtual file to virtual file using sendfile</t>
+  </si>
+  <si>
+    <t>Copy virtual file to real file using sendfile</t>
   </si>
   <si>
     <t>Field as string</t>
@@ -542,7 +800,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -557,7 +815,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -572,7 +830,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -588,7 +846,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778105145" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -597,7 +855,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -610,7 +868,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -621,7 +879,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -632,7 +890,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -643,7 +901,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -654,7 +912,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -665,7 +923,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -676,7 +934,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -687,13 +945,24 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -709,7 +978,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
+          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
         </ext>
       </extLst>
     </border>
@@ -728,7 +997,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145">
+          <pm:border xmlns:pm="smNativeData" id="1778192348">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -750,7 +1019,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145">
+          <pm:border xmlns:pm="smNativeData" id="1778192348">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -774,7 +1043,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145">
+          <pm:border xmlns:pm="smNativeData" id="1778192348">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -798,7 +1067,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145">
+          <pm:border xmlns:pm="smNativeData" id="1778192348">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -822,7 +1091,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
+          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
         </ext>
       </extLst>
     </border>
@@ -841,7 +1110,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
+          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
         </ext>
       </extLst>
     </border>
@@ -860,7 +1129,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
+          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
         </ext>
       </extLst>
     </border>
@@ -879,7 +1148,26 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778105145"/>
+          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
         </ext>
       </extLst>
     </border>
@@ -935,13 +1223,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="37">
+  <dxfs count="42">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -954,7 +1242,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -965,7 +1253,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -978,7 +1266,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -989,7 +1277,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1002,7 +1290,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1013,7 +1301,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1026,7 +1314,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1037,7 +1325,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1050,7 +1338,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1061,7 +1349,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1074,7 +1362,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1085,7 +1373,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1098,7 +1386,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1109,7 +1397,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1122,7 +1410,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1133,7 +1421,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1146,7 +1434,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1157,7 +1445,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1170,7 +1458,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1181,7 +1469,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1194,7 +1482,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1205,7 +1493,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1218,7 +1506,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1229,7 +1517,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1242,7 +1530,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1253,7 +1541,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1266,7 +1554,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1277,7 +1565,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1290,7 +1578,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1301,7 +1589,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1314,7 +1602,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1325,7 +1613,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1338,7 +1626,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1349,7 +1637,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1362,7 +1650,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1373,7 +1661,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1386,7 +1674,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1397,7 +1685,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1410,7 +1698,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1421,7 +1709,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1434,7 +1722,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1445,7 +1733,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1458,7 +1746,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1469,7 +1757,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1482,7 +1770,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1493,7 +1781,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1506,7 +1794,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1517,7 +1805,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1530,7 +1818,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1541,7 +1829,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1554,7 +1842,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1565,7 +1853,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1578,7 +1866,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1589,7 +1877,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1602,7 +1890,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1613,7 +1901,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1626,7 +1914,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1637,7 +1925,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1650,7 +1938,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1661,7 +1949,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1674,7 +1962,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1685,7 +1973,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1698,7 +1986,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1709,7 +1997,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1722,7 +2010,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1733,7 +2021,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1746,7 +2034,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1757,7 +2045,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1770,7 +2058,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1781,7 +2069,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1794,7 +2082,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1805,7 +2093,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778105145" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1818,7 +2106,127 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778105145" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1828,10 +2236,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778105145" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778192348" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778105145" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778192348" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3261,7 +3669,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3270,14 +3678,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3367,7 +3775,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3378,14 +3786,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3396,10 +3804,10 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B112"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
-    <col min="1" max="1" width="55.482143" customWidth="1" style="0"/>
+    <col min="1" max="1" width="64.723214" customWidth="1" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3540,7 +3948,9 @@
       <c r="A20" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="B20" s="10"/>
+      <c r="B20" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
@@ -3583,26 +3993,597 @@
         <v>134</v>
       </c>
       <c r="B26" s="10"/>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B30" s="10"/>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B31" s="10"/>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B33" s="10"/>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B34" s="10"/>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B35" s="10"/>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" s="10"/>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B38" s="10"/>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B39" s="10"/>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B40" s="10"/>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B41" s="10"/>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B42" s="10"/>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="B43" s="10"/>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="B44" s="10"/>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B45" s="10"/>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="B46" s="10"/>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B47" s="10"/>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B48" s="10"/>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="B49" s="10"/>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B50" s="10"/>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B51" s="10"/>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="B52" s="10"/>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="B53" s="10"/>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B54" s="10"/>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B55" s="10"/>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B56" s="10"/>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="B57" s="10"/>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="B58" s="10"/>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="B59" s="10"/>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B60" s="10"/>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="B61" s="10"/>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B62" s="10"/>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="B63" s="10"/>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="B64" s="10"/>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B65" s="10"/>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B66" s="10"/>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B67" s="10"/>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B68" s="10"/>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B69" s="10"/>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="B70" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B71" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="B72" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B73" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B74" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="B75" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B76" s="10"/>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B77" s="10"/>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B78" s="10"/>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B79" s="10"/>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B80" s="10"/>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="B81" s="10"/>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="B82" s="10"/>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="B83" s="10"/>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B84" s="10"/>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B85" s="10"/>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B86" s="10"/>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B87" s="10"/>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="B88" s="10"/>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="B89" s="10"/>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="B90" s="10"/>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="B91" s="10"/>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="B92" s="10"/>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B93" s="10"/>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="B94" s="10"/>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B95" s="10"/>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="B96" s="10"/>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B97" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="B98" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B99" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B100" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B101" s="10"/>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B102" s="10"/>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B103" s="10"/>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="B104" s="10"/>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B105" s="10"/>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B106" s="10"/>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="B107" s="10"/>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="B108" s="10"/>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="B109" s="10"/>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="B110" s="10"/>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="B111" s="10"/>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="B112" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B3:B26">
+  <conditionalFormatting sqref="B73:B112">
     <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B43:B72">
+    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:B72">
+    <cfRule type="cellIs" dxfId="37" priority="3" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27:B42">
+    <cfRule type="cellIs" dxfId="38" priority="4" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27:B42">
+    <cfRule type="cellIs" dxfId="39" priority="5" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B3:B26">
-    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="6" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B26">
+    <cfRule type="cellIs" dxfId="41" priority="7" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3613,14 +4594,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3649,55 +4630,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>135</v>
+        <v>221</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>136</v>
+        <v>222</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>137</v>
+        <v>223</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>138</v>
+        <v>224</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>139</v>
+        <v>225</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>140</v>
+        <v>226</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>141</v>
+        <v>227</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>142</v>
+        <v>228</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>143</v>
+        <v>229</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -3709,7 +4690,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3720,14 +4701,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3756,19 +4737,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>144</v>
+        <v>230</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>145</v>
+        <v>231</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>146</v>
+        <v>232</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -3780,7 +4761,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3791,14 +4772,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3828,7 +4809,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>147</v>
+        <v>233</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3836,7 +4817,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>148</v>
+        <v>234</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3844,7 +4825,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>149</v>
+        <v>235</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3852,7 +4833,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>150</v>
+        <v>236</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -3860,7 +4841,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>151</v>
+        <v>237</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -3868,7 +4849,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>152</v>
+        <v>238</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -3876,7 +4857,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>153</v>
+        <v>239</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -3884,7 +4865,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>154</v>
+        <v>240</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -3892,7 +4873,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>155</v>
+        <v>241</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -3900,7 +4881,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>156</v>
+        <v>242</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -3908,7 +4889,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>157</v>
+        <v>243</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -3916,7 +4897,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>158</v>
+        <v>244</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -3930,7 +4911,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3939,14 +4920,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4030,7 +5011,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4041,14 +5022,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4139,7 +5120,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4150,14 +5131,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4196,7 +5177,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4207,14 +5188,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4553,7 +5534,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4564,14 +5545,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4642,7 +5623,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4653,14 +5634,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4741,7 +5722,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4752,14 +5733,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4871,7 +5852,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4882,14 +5863,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4964,7 +5945,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778105145" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4975,14 +5956,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778105145" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778105145" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added tests involving std.fs.File (#893)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778192348" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778192348" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778192348" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778192348"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778280406" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778280406" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778280406" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778280406"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="245">
   <si>
     <t>Context</t>
   </si>
@@ -800,7 +800,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -815,7 +815,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -830,7 +830,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -846,7 +846,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778192348" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -855,7 +855,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -868,7 +868,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -879,7 +879,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -890,7 +890,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -901,7 +901,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -912,7 +912,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -923,7 +923,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -934,35 +934,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFB3B3"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -978,7 +956,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
+          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
         </ext>
       </extLst>
     </border>
@@ -997,7 +975,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348">
+          <pm:border xmlns:pm="smNativeData" id="1778280406">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1019,7 +997,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348">
+          <pm:border xmlns:pm="smNativeData" id="1778280406">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1043,7 +1021,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348">
+          <pm:border xmlns:pm="smNativeData" id="1778280406">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1067,7 +1045,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348">
+          <pm:border xmlns:pm="smNativeData" id="1778280406">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1091,7 +1069,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
+          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
         </ext>
       </extLst>
     </border>
@@ -1110,7 +1088,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
+          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
         </ext>
       </extLst>
     </border>
@@ -1129,45 +1107,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778192348"/>
+          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
         </ext>
       </extLst>
     </border>
@@ -1180,7 +1120,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1214,6 +1154,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -1229,7 +1172,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1242,7 +1185,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1253,7 +1196,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1266,7 +1209,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1277,7 +1220,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1290,7 +1233,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1301,7 +1244,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1314,7 +1257,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1325,7 +1268,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1338,7 +1281,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1349,7 +1292,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1362,7 +1305,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1373,7 +1316,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1386,7 +1329,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1397,7 +1340,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1410,7 +1353,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1421,7 +1364,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1434,7 +1377,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1445,7 +1388,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1458,7 +1401,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1469,7 +1412,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1482,7 +1425,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1493,7 +1436,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1506,7 +1449,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1517,7 +1460,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1530,7 +1473,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1541,7 +1484,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1554,7 +1497,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1565,7 +1508,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1578,7 +1521,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1589,7 +1532,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1602,7 +1545,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1613,7 +1556,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1626,7 +1569,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1637,7 +1580,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1650,7 +1593,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1661,7 +1604,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1674,7 +1617,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1685,7 +1628,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1698,7 +1641,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1709,7 +1652,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1722,7 +1665,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1733,7 +1676,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1746,7 +1689,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1757,7 +1700,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1770,7 +1713,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1781,7 +1724,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1794,7 +1737,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1805,7 +1748,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1818,7 +1761,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1829,7 +1772,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1842,7 +1785,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1853,7 +1796,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1866,7 +1809,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1877,7 +1820,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1890,7 +1833,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1901,7 +1844,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1914,7 +1857,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1925,7 +1868,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1938,7 +1881,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1949,7 +1892,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1962,7 +1905,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1973,7 +1916,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1986,7 +1929,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1997,7 +1940,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2010,7 +1953,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2021,7 +1964,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2034,7 +1977,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2045,7 +1988,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2058,7 +2001,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2069,7 +2012,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2082,7 +2025,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2093,7 +2036,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2106,7 +2049,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2117,7 +2060,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2130,7 +2073,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2141,7 +2084,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2154,7 +2097,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2165,7 +2108,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2178,7 +2121,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2189,7 +2132,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2202,7 +2145,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2213,7 +2156,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778192348" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2226,7 +2169,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778192348" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2236,10 +2179,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778192348" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778280406" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778192348" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778280406" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3669,7 +3612,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3678,14 +3621,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3775,7 +3718,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3786,14 +3729,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3804,7 +3747,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B112"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="64.723214" customWidth="1" style="0"/>
@@ -3824,13 +3767,17 @@
       <c r="A3" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="10"/>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
@@ -3892,13 +3839,20 @@
       <c r="A12" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="B12" s="10"/>
-    </row>
-    <row r="13" spans="1:2">
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
@@ -3956,13 +3910,17 @@
       <c r="A21" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="B21" s="10"/>
+      <c r="B21" s="10" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="B22" s="10"/>
+      <c r="B22" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
@@ -4022,7 +3980,9 @@
       <c r="A30" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="B30" s="10"/>
+      <c r="B30" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="9" t="s">
@@ -4064,11 +4024,16 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:4">
       <c r="A37" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B37" s="10"/>
+      <c r="B37" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="9" t="s">
@@ -4583,7 +4548,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4594,14 +4559,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4690,7 +4655,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4701,14 +4666,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4761,7 +4726,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4772,14 +4737,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4911,7 +4876,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4920,14 +4885,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5011,7 +4976,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5022,14 +4987,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5120,7 +5085,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5131,14 +5096,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5177,7 +5142,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5188,14 +5153,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5534,7 +5499,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5545,14 +5510,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5623,7 +5588,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5634,14 +5599,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5722,7 +5687,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5733,14 +5698,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5852,7 +5817,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5863,14 +5828,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5945,7 +5910,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778192348" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5956,14 +5921,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778192348" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778192348" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added directory tests *#918)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778280406" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778280406" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778280406" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778280406"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778629906" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778629906" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778629906" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778629906"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="245">
   <si>
     <t>Context</t>
   </si>
@@ -683,7 +683,7 @@
     <t>Ignore offset to WriteFile when stream is unseekable</t>
   </si>
   <si>
-    <t>Copy read file to virtual file</t>
+    <t>Copy real file to virtual file</t>
   </si>
   <si>
     <t>Copy virtual file to virtual file</t>
@@ -800,7 +800,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -815,7 +815,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -830,7 +830,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -846,7 +846,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778280406" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -868,7 +868,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -879,7 +879,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -890,7 +890,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -901,7 +901,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -912,7 +912,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -923,7 +923,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -934,7 +934,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -956,7 +956,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
+          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
         </ext>
       </extLst>
     </border>
@@ -975,7 +975,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406">
+          <pm:border xmlns:pm="smNativeData" id="1778629906">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -997,7 +997,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406">
+          <pm:border xmlns:pm="smNativeData" id="1778629906">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1021,7 +1021,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406">
+          <pm:border xmlns:pm="smNativeData" id="1778629906">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1045,7 +1045,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406">
+          <pm:border xmlns:pm="smNativeData" id="1778629906">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1069,7 +1069,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
+          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
         </ext>
       </extLst>
     </border>
@@ -1088,7 +1088,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
+          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
         </ext>
       </extLst>
     </border>
@@ -1107,7 +1107,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778280406"/>
+          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
         </ext>
       </extLst>
     </border>
@@ -1120,7 +1120,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1154,9 +1154,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -1172,7 +1169,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1185,7 +1182,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1196,7 +1193,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1209,7 +1206,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1220,7 +1217,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1233,7 +1230,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1244,7 +1241,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1257,7 +1254,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1268,7 +1265,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1281,7 +1278,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1292,7 +1289,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1305,7 +1302,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1316,7 +1313,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1329,7 +1326,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1340,7 +1337,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1353,7 +1350,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1364,7 +1361,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1377,7 +1374,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1388,7 +1385,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1401,7 +1398,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1412,7 +1409,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1425,7 +1422,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1436,7 +1433,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1449,7 +1446,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1460,7 +1457,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1473,7 +1470,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1484,7 +1481,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1497,7 +1494,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1508,7 +1505,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1521,7 +1518,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1532,7 +1529,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1545,7 +1542,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1556,7 +1553,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1569,7 +1566,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1580,7 +1577,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1593,7 +1590,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1604,7 +1601,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1617,7 +1614,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1628,7 +1625,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1641,7 +1638,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1652,7 +1649,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1665,7 +1662,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1676,7 +1673,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1689,7 +1686,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1700,7 +1697,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1713,7 +1710,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1724,7 +1721,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1737,7 +1734,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1748,7 +1745,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1761,7 +1758,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1772,7 +1769,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1785,7 +1782,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1796,7 +1793,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1809,7 +1806,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1820,7 +1817,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1833,7 +1830,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1844,7 +1841,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1857,7 +1854,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1868,7 +1865,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1881,7 +1878,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1892,7 +1889,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1905,7 +1902,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1916,7 +1913,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1929,7 +1926,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1940,7 +1937,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1953,7 +1950,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1964,7 +1961,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1977,7 +1974,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1988,7 +1985,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2001,7 +1998,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2012,7 +2009,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2025,7 +2022,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2036,7 +2033,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2049,7 +2046,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2060,7 +2057,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2073,7 +2070,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2084,7 +2081,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2097,7 +2094,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2108,7 +2105,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2121,7 +2118,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2132,7 +2129,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2145,7 +2142,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2156,7 +2153,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778280406" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2169,7 +2166,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778280406" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2179,10 +2176,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778280406" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778629906" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778280406" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778629906" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3612,7 +3609,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3621,14 +3618,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3718,7 +3715,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3729,14 +3726,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3816,7 +3813,7 @@
         <v>117</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -3850,7 +3847,7 @@
       <c r="B13" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="13" t="s">
         <v>92</v>
       </c>
     </row>
@@ -3906,12 +3903,15 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
         <v>129</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -4029,9 +4029,9 @@
         <v>145</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D37" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D37" s="13" t="s">
         <v>92</v>
       </c>
     </row>
@@ -4147,49 +4147,65 @@
       <c r="A56" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="B56" s="10"/>
+      <c r="B56" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="B57" s="10"/>
+      <c r="B57" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="B58" s="10"/>
+      <c r="B58" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="B59" s="10"/>
+      <c r="B59" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="B60" s="10"/>
+      <c r="B60" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="B61" s="10"/>
+      <c r="B61" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="B62" s="10"/>
+      <c r="B62" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B63" s="10"/>
+      <c r="B63" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="9" t="s">
@@ -4333,7 +4349,9 @@
       <c r="A85" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="B85" s="10"/>
+      <c r="B85" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="9" t="s">
@@ -4351,7 +4369,9 @@
       <c r="A88" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="B88" s="10"/>
+      <c r="B88" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="9" t="s">
@@ -4473,37 +4493,49 @@
       <c r="A107" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="B107" s="10"/>
+      <c r="B107" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="B108" s="10"/>
+      <c r="B108" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B109" s="10"/>
+      <c r="B109" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="B110" s="10"/>
+      <c r="B110" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="B111" s="10"/>
+      <c r="B111" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="B112" s="10"/>
+      <c r="B112" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4548,7 +4580,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4559,14 +4591,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4655,7 +4687,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4666,14 +4698,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4726,7 +4758,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4737,14 +4769,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4876,7 +4908,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4885,14 +4917,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4976,7 +5008,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4987,14 +5019,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5085,7 +5117,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5096,14 +5128,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5142,7 +5174,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5153,14 +5185,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5499,7 +5531,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5510,14 +5542,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5588,7 +5620,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5599,14 +5631,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5687,7 +5719,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5698,14 +5730,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5817,7 +5849,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5828,14 +5860,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5910,7 +5942,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778280406" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5921,14 +5953,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778280406" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778280406" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added tests related to file time (#918)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778629906" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778629906" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778629906" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778629906"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778694661" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778694661" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778694661" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778694661"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="246">
   <si>
     <t>Context</t>
   </si>
@@ -476,7 +476,7 @@
     <t>Decompress gzip file</t>
   </si>
   <si>
-    <t>Get stats of Uint8Array</t>
+    <t>Get stats of virtual file</t>
   </si>
   <si>
     <t>Get stats of opened file using posix function</t>
@@ -500,7 +500,7 @@
     <t>Set access and last modified time of opened file using futime</t>
   </si>
   <si>
-    <t>Set access and last modified time of file using posix function</t>
+    <t>Set access and last modified time of file using posix function with ns precision</t>
   </si>
   <si>
     <t>Set access and last modified time of file using utime</t>
@@ -663,6 +663,9 @@
   </si>
   <si>
     <t>Remove file in file system using posix function</t>
+  </si>
+  <si>
+    <t>Update mtime/atime of file in file system using posix function</t>
   </si>
   <si>
     <t>Scan directory in file system using posix function</t>
@@ -800,7 +803,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -815,7 +818,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -830,7 +833,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -846,7 +849,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778629906" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -855,7 +858,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -868,7 +871,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -879,7 +882,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -890,7 +893,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -901,7 +904,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -912,7 +915,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -923,7 +926,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -934,13 +937,24 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -956,7 +970,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
+          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
         </ext>
       </extLst>
     </border>
@@ -975,7 +989,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906">
+          <pm:border xmlns:pm="smNativeData" id="1778694661">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -997,7 +1011,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906">
+          <pm:border xmlns:pm="smNativeData" id="1778694661">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1021,7 +1035,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906">
+          <pm:border xmlns:pm="smNativeData" id="1778694661">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1045,7 +1059,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906">
+          <pm:border xmlns:pm="smNativeData" id="1778694661">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1069,7 +1083,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
+          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
         </ext>
       </extLst>
     </border>
@@ -1088,7 +1102,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
+          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
         </ext>
       </extLst>
     </border>
@@ -1107,7 +1121,26 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778629906"/>
+          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
         </ext>
       </extLst>
     </border>
@@ -1120,7 +1153,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1154,6 +1187,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -1169,7 +1205,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1182,7 +1218,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1193,7 +1229,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1206,7 +1242,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1217,7 +1253,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1230,7 +1266,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1241,7 +1277,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1254,7 +1290,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1265,7 +1301,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1278,7 +1314,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1289,7 +1325,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1302,7 +1338,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1313,7 +1349,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1326,7 +1362,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1337,7 +1373,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1350,7 +1386,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1361,7 +1397,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1374,7 +1410,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1385,7 +1421,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1398,7 +1434,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1409,7 +1445,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1422,7 +1458,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1433,7 +1469,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1446,7 +1482,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1457,7 +1493,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1470,7 +1506,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1481,7 +1517,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1494,7 +1530,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1505,7 +1541,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1518,7 +1554,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1529,7 +1565,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1542,7 +1578,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1553,7 +1589,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1566,7 +1602,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1577,7 +1613,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1590,7 +1626,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1601,7 +1637,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1614,7 +1650,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1625,7 +1661,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1638,7 +1674,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1649,7 +1685,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1662,7 +1698,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1673,7 +1709,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1686,7 +1722,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1697,7 +1733,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1710,7 +1746,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1721,7 +1757,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1734,7 +1770,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1745,7 +1781,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1758,7 +1794,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1769,7 +1805,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1782,7 +1818,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1793,7 +1829,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1806,7 +1842,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1817,7 +1853,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1830,7 +1866,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1841,7 +1877,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1854,7 +1890,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1865,7 +1901,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1878,7 +1914,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1889,7 +1925,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1902,7 +1938,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1913,7 +1949,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1926,7 +1962,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1937,7 +1973,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1950,7 +1986,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1961,7 +1997,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1974,7 +2010,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1985,7 +2021,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1998,7 +2034,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2009,7 +2045,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2022,7 +2058,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2033,7 +2069,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2046,7 +2082,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2057,7 +2093,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2070,7 +2106,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2081,7 +2117,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2094,7 +2130,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2105,7 +2141,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2118,7 +2154,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2129,7 +2165,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2142,7 +2178,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2153,7 +2189,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778629906" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2166,7 +2202,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778629906" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2176,10 +2212,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778629906" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778694661" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778629906" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1778694661" count="7">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3609,7 +3645,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3618,14 +3654,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3715,7 +3751,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3726,14 +3762,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3744,10 +3780,10 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D112"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
-    <col min="1" max="1" width="64.723214" customWidth="1" style="0"/>
+    <col min="1" max="1" width="68.473214" customWidth="1" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3988,7 +4024,9 @@
       <c r="A31" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="B31" s="10"/>
+      <c r="B31" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="9" t="s">
@@ -4002,19 +4040,25 @@
       <c r="A33" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="B33" s="10"/>
+      <c r="B33" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="B34" s="10"/>
+      <c r="B34" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="B35" s="10"/>
+      <c r="B35" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="9" t="s">
@@ -4035,29 +4079,38 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:4">
       <c r="A38" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B38" s="10"/>
+      <c r="B38" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38" s="15"/>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B39" s="10"/>
+      <c r="B39" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="B40" s="10"/>
+      <c r="B40" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="B41" s="10"/>
+      <c r="B41" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="9" t="s">
@@ -4075,7 +4128,9 @@
       <c r="A44" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B44" s="10"/>
+      <c r="B44" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="9" t="s">
@@ -4087,19 +4142,25 @@
       <c r="A46" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="B46" s="10"/>
+      <c r="B46" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="B47" s="10"/>
+      <c r="B47" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="B48" s="10"/>
+      <c r="B48" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="9" t="s">
@@ -4135,13 +4196,17 @@
       <c r="A54" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="B54" s="10"/>
+      <c r="B54" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B55" s="10"/>
+      <c r="B55" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="9" t="s">
@@ -4383,7 +4448,9 @@
       <c r="A90" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="B90" s="10"/>
+      <c r="B90" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
@@ -4395,7 +4462,9 @@
       <c r="A92" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B92" s="10"/>
+      <c r="B92" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
@@ -4407,7 +4476,9 @@
       <c r="A94" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="B94" s="10"/>
+      <c r="B94" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
@@ -4457,13 +4528,17 @@
       <c r="A101" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B101" s="10"/>
+      <c r="B101" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="B102" s="10"/>
+      <c r="B102" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="9" t="s">
@@ -4493,9 +4568,7 @@
       <c r="A107" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="B107" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B107" s="10"/>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="9" t="s">
@@ -4534,6 +4607,14 @@
         <v>220</v>
       </c>
       <c r="B112" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="B113" s="10" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4542,7 +4623,7 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B73:B112">
+  <conditionalFormatting sqref="B73:B113">
     <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
@@ -4580,7 +4661,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4591,14 +4672,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4627,55 +4708,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -4687,7 +4768,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4698,14 +4779,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4734,19 +4815,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -4758,7 +4839,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4769,14 +4850,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4806,7 +4887,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4814,7 +4895,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4822,7 +4903,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4830,7 +4911,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -4838,7 +4919,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4846,7 +4927,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -4854,7 +4935,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -4862,7 +4943,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -4870,7 +4951,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -4878,7 +4959,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -4886,7 +4967,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -4894,7 +4975,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -4908,7 +4989,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4917,14 +4998,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5008,7 +5089,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5019,14 +5100,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5117,7 +5198,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5128,14 +5209,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5174,7 +5255,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5185,14 +5266,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5531,7 +5612,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5542,14 +5623,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5620,7 +5701,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5631,14 +5712,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5719,7 +5800,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5730,14 +5811,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5849,7 +5930,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5860,14 +5941,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5942,7 +6023,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778629906" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5953,14 +6034,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778629906" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778629906" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added tests related to file locking (#918)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778694661" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778694661" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778694661" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778694661"/>
+      <pm:revision xmlns:pm="smNativeData" day="1779145613" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1779145613" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1779145613" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1779145613"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="247">
   <si>
     <t>Context</t>
   </si>
@@ -521,7 +521,10 @@
     <t>Perform datasync operation using posix function</t>
   </si>
   <si>
-    <t>Perform allocate operation using posix function</t>
+    <t>Perform advise operation using posix function</t>
+  </si>
+  <si>
+    <t>Fail to perform allocate operation using posix function</t>
   </si>
   <si>
     <t>Open file in directory</t>
@@ -557,19 +560,19 @@
     <t>Create symlink</t>
   </si>
   <si>
-    <t>Create symlink in directory</t>
-  </si>
-  <si>
-    <t>Create symlink using posix function</t>
-  </si>
-  <si>
-    <t>Create symlink in directory using posix function</t>
-  </si>
-  <si>
-    <t>Create symlink in file system using posix function</t>
-  </si>
-  <si>
-    <t>Create symlink using win32 function</t>
+    <t>Fail to create symlink in directory</t>
+  </si>
+  <si>
+    <t>Fail to create symlink using posix function</t>
+  </si>
+  <si>
+    <t>Fail to create symlink in directory using posix function</t>
+  </si>
+  <si>
+    <t>Fail to create symlink in file system using posix function</t>
+  </si>
+  <si>
+    <t>Fail to create symlink using win32 function</t>
   </si>
   <si>
     <t>Open and read from file using pread</t>
@@ -593,7 +596,10 @@
     <t>Set lock on file</t>
   </si>
   <si>
-    <t>Get lock on file using fcntl</t>
+    <t>Set lock on file using fcntl</t>
+  </si>
+  <si>
+    <t>Fail to get lock on file using fcntl</t>
   </si>
   <si>
     <t>Set lock on file using posix function</t>
@@ -614,9 +620,6 @@
     <t>Scan variables from stdin using scanf</t>
   </si>
   <si>
-    <t>Scan variables from web stream using scanf</t>
-  </si>
-  <si>
     <t>Get characters from a file using fgetc</t>
   </si>
   <si>
@@ -671,7 +674,7 @@
     <t>Scan directory in file system using posix function</t>
   </si>
   <si>
-    <t>Read link using posix function</t>
+    <t>Fail to read link using posix function</t>
   </si>
   <si>
     <t>Fail to convert to file when useRedirection is false</t>
@@ -803,7 +806,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -818,7 +821,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -833,7 +836,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -849,7 +852,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778694661" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -858,7 +861,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -871,7 +874,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -882,7 +885,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -893,7 +896,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -904,7 +907,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -915,7 +918,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -926,7 +929,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5C5CFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -937,7 +951,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -948,13 +962,24 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5C5CFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -970,7 +995,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
+          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
         </ext>
       </extLst>
     </border>
@@ -989,7 +1014,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661">
+          <pm:border xmlns:pm="smNativeData" id="1779145613">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1011,7 +1036,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661">
+          <pm:border xmlns:pm="smNativeData" id="1779145613">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1035,7 +1060,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661">
+          <pm:border xmlns:pm="smNativeData" id="1779145613">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1059,7 +1084,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661">
+          <pm:border xmlns:pm="smNativeData" id="1779145613">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1083,7 +1108,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
+          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
         </ext>
       </extLst>
     </border>
@@ -1102,7 +1127,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
+          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
         </ext>
       </extLst>
     </border>
@@ -1121,7 +1146,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
+          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
         </ext>
       </extLst>
     </border>
@@ -1140,7 +1165,45 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778694661"/>
+          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
         </ext>
       </extLst>
     </border>
@@ -1153,7 +1216,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1187,6 +1250,15 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1205,7 +1277,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1218,7 +1290,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1229,7 +1301,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1242,7 +1314,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1253,7 +1325,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1266,7 +1338,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1277,7 +1349,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1290,7 +1362,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1301,7 +1373,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1314,7 +1386,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1325,7 +1397,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1338,7 +1410,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1349,7 +1421,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1362,7 +1434,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1373,7 +1445,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1386,7 +1458,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1397,7 +1469,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1410,7 +1482,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1421,7 +1493,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1434,7 +1506,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1445,7 +1517,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1458,7 +1530,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1469,7 +1541,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1482,7 +1554,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1493,7 +1565,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1506,7 +1578,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1517,7 +1589,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1530,7 +1602,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1541,7 +1613,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1554,7 +1626,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1565,7 +1637,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1578,7 +1650,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1589,7 +1661,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1602,7 +1674,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1613,7 +1685,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1626,7 +1698,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1637,7 +1709,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1650,7 +1722,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1661,7 +1733,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1674,7 +1746,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1685,7 +1757,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1698,7 +1770,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1709,7 +1781,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1722,7 +1794,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1733,7 +1805,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1746,7 +1818,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1757,7 +1829,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1770,7 +1842,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1781,7 +1853,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1794,7 +1866,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1805,7 +1877,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1818,7 +1890,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1829,7 +1901,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1842,7 +1914,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1853,7 +1925,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1866,7 +1938,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1877,7 +1949,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1890,7 +1962,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1901,7 +1973,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1914,7 +1986,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1925,7 +1997,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1938,7 +2010,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1949,7 +2021,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1962,7 +2034,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1973,7 +2045,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1986,7 +2058,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1997,7 +2069,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2010,7 +2082,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2021,7 +2093,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2034,7 +2106,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2045,7 +2117,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2058,7 +2130,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2069,7 +2141,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2082,7 +2154,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2093,7 +2165,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2106,7 +2178,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2117,7 +2189,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2130,7 +2202,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2141,7 +2213,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2154,7 +2226,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2165,7 +2237,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2178,7 +2250,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2189,7 +2261,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778694661" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2202,7 +2274,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778694661" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2212,10 +2284,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778694661" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1779145613" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778694661" count="7">
+      <pm:colors xmlns:pm="smNativeData" id="1779145613" count="8">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -2223,6 +2295,7 @@
         <pm:color name="Color 28" rgb="808080"/>
         <pm:color name="Color 29" rgb="FFB3B3"/>
         <pm:color name="Color 30" rgb="FFFF9E"/>
+        <pm:color name="Color 31" rgb="5C5CFF"/>
       </pm:colors>
     </ext>
   </extLst>
@@ -3645,7 +3718,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3654,14 +3727,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3751,7 +3824,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3762,14 +3835,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3780,10 +3853,11 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D114"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="68.473214" customWidth="1" style="0"/>
+    <col min="4" max="4" width="12.419643" customWidth="1" style="18"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3907,13 +3981,13 @@
       <c r="A16" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="15"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="B17" s="10"/>
+      <c r="B17" s="15"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
@@ -3986,7 +4060,7 @@
       <c r="A26" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B26" s="10"/>
+      <c r="B26" s="15"/>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="9" t="s">
@@ -4086,7 +4160,7 @@
       <c r="B38" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D38" s="15"/>
+      <c r="D38" s="13"/>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
@@ -4116,13 +4190,13 @@
       <c r="A42" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="B42" s="10"/>
+      <c r="B42" s="15"/>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="B43" s="10"/>
+      <c r="B43" s="15"/>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="9" t="s">
@@ -4136,7 +4210,7 @@
       <c r="A45" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="B45" s="10"/>
+      <c r="B45" s="15"/>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="9" t="s">
@@ -4166,31 +4240,44 @@
       <c r="A49" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B49" s="10"/>
-    </row>
-    <row r="50" spans="1:2">
+      <c r="B49" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="B50" s="10"/>
+      <c r="B50" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50" s="13" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="B51" s="10"/>
+      <c r="B51" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="B52" s="10"/>
+      <c r="B52" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="B53" s="10"/>
+      <c r="B53" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="9" t="s">
@@ -4276,45 +4363,55 @@
       <c r="A64" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B64" s="10"/>
+      <c r="B64" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="B65" s="10"/>
+      <c r="B65" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="B66" s="10"/>
+      <c r="B66" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="B67" s="10"/>
+      <c r="B67" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="B68" s="10"/>
+      <c r="B68" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="B69" s="10"/>
+      <c r="B69" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="B70" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B70" s="17"/>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="9" t="s">
@@ -4360,55 +4457,82 @@
       <c r="A76" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="B76" s="10"/>
+      <c r="B76" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B77" s="10"/>
+      <c r="B77" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B78" s="10"/>
+      <c r="B78" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="B79" s="10"/>
+      <c r="B79" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B80" s="10"/>
-    </row>
-    <row r="81" spans="1:2">
+      <c r="B80" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
       <c r="A81" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="B81" s="10"/>
-    </row>
-    <row r="82" spans="1:2">
+      <c r="B81" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D81" s="18" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
       <c r="A82" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="B82" s="10"/>
-    </row>
-    <row r="83" spans="1:2">
+      <c r="B82" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D82" s="16" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
       <c r="A83" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="B83" s="10"/>
+      <c r="B83" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D83" s="16" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="B84" s="10"/>
+      <c r="B84" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="9" t="s">
@@ -4422,13 +4546,18 @@
       <c r="A86" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="B86" s="10"/>
-    </row>
-    <row r="87" spans="1:2">
+      <c r="B86" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
       <c r="A87" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B87" s="10"/>
+      <c r="B87" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87" s="16"/>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="9" t="s">
@@ -4442,49 +4571,51 @@
       <c r="A89" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B89" s="10"/>
+      <c r="B89" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="B90" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B90" s="15"/>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="B91" s="10"/>
+      <c r="B91" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B92" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B92" s="15"/>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="B93" s="10"/>
+      <c r="B93" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="B94" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B94" s="15"/>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="B95" s="10"/>
+      <c r="B95" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="9" t="s">
@@ -4496,9 +4627,7 @@
       <c r="A97" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="B97" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B97" s="10"/>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="9" t="s">
@@ -4544,39 +4673,53 @@
       <c r="A103" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="B103" s="10"/>
-    </row>
-    <row r="104" spans="1:2">
+      <c r="B103" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
       <c r="A104" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="B104" s="10"/>
-    </row>
-    <row r="105" spans="1:2">
+      <c r="B104" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104" s="16"/>
+    </row>
+    <row r="105" spans="1:4">
       <c r="A105" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="B105" s="10"/>
-    </row>
-    <row r="106" spans="1:2">
+      <c r="B105" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D105" s="16"/>
+    </row>
+    <row r="106" spans="1:4">
       <c r="A106" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="B106" s="10"/>
-    </row>
-    <row r="107" spans="1:2">
+      <c r="B106" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D106" s="16"/>
+    </row>
+    <row r="107" spans="1:4">
       <c r="A107" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="B107" s="10"/>
+      <c r="B107" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D107" s="16" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="B108" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B108" s="15"/>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
@@ -4615,6 +4758,14 @@
         <v>221</v>
       </c>
       <c r="B113" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="B114" s="10" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4623,17 +4774,17 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B73:B113">
+  <conditionalFormatting sqref="B74:B114">
     <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43:B72">
+  <conditionalFormatting sqref="B43:B73">
     <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43:B72">
+  <conditionalFormatting sqref="B43:B73">
     <cfRule type="cellIs" dxfId="37" priority="3" operator="equal">
       <formula>N</formula>
     </cfRule>
@@ -4661,7 +4812,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4672,14 +4823,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4708,55 +4859,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -4768,7 +4919,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4779,14 +4930,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4815,19 +4966,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -4839,7 +4990,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4850,14 +5001,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4887,7 +5038,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4895,7 +5046,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4903,7 +5054,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4911,7 +5062,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -4919,7 +5070,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4927,7 +5078,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -4935,7 +5086,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -4943,7 +5094,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -4951,7 +5102,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -4959,7 +5110,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -4967,7 +5118,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -4975,7 +5126,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -4989,7 +5140,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4998,14 +5149,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5089,7 +5240,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5100,14 +5251,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5198,7 +5349,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5209,14 +5360,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5255,7 +5406,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5266,14 +5417,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5612,7 +5763,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5623,14 +5774,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5701,7 +5852,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5712,14 +5863,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5800,7 +5951,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5811,14 +5962,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5930,7 +6081,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5941,14 +6092,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6023,7 +6174,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778694661" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6034,14 +6185,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778694661" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778694661" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added yet another image processing test (#928)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="10" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
+    <workbookView activeTab="11" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -19,24 +19,25 @@
     <sheet name="Package manager" sheetId="9" r:id="rId12"/>
     <sheet name="Iterator" sheetId="10" r:id="rId13"/>
     <sheet name="Stream handling" sheetId="11" r:id="rId14"/>
-    <sheet name="Metadata" sheetId="12" r:id="rId15"/>
-    <sheet name="Options" sheetId="13" r:id="rId16"/>
-    <sheet name="JS-compat objects" sheetId="14" r:id="rId17"/>
+    <sheet name="Image processing" sheetId="12" r:id="rId15"/>
+    <sheet name="Metatypes" sheetId="13" r:id="rId16"/>
+    <sheet name="Options" sheetId="14" r:id="rId17"/>
+    <sheet name="JS-compat objects" sheetId="15" r:id="rId18"/>
   </sheets>
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1779145613" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1779145613" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1779145613" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1779145613"/>
+      <pm:revision xmlns:pm="smNativeData" day="1779342094" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1779342094" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1779342094" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1779342094"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="262">
   <si>
     <t>Context</t>
   </si>
@@ -599,7 +600,7 @@
     <t>Set lock on file using fcntl</t>
   </si>
   <si>
-    <t>Fail to get lock on file using fcntl</t>
+    <t>Get lock on file using fcntl</t>
   </si>
   <si>
     <t>Set lock on file using posix function</t>
@@ -608,6 +609,9 @@
     <t>Set lock on file inside thread</t>
   </si>
   <si>
+    <t>Set non-blocking flag using fctnl</t>
+  </si>
+  <si>
     <t>Read lines from file using fgets</t>
   </si>
   <si>
@@ -650,7 +654,7 @@
     <t>Make directory in directory</t>
   </si>
   <si>
-    <t>Read files using poll function</t>
+    <t>Fail to poll file</t>
   </si>
   <si>
     <t>Redirect io from dynamically linked library</t>
@@ -707,6 +711,39 @@
     <t>Copy virtual file to real file using sendfile</t>
   </si>
   <si>
+    <t>Get file descriptor using libc function</t>
+  </si>
+  <si>
+    <t>Check if stream is terminal using libc function</t>
+  </si>
+  <si>
+    <t>Get terminal name using libc function</t>
+  </si>
+  <si>
+    <t>Basic rendering</t>
+  </si>
+  <si>
+    <t>Resizing</t>
+  </si>
+  <si>
+    <t>Sepia</t>
+  </si>
+  <si>
+    <t>Circle pattern</t>
+  </si>
+  <si>
+    <t>Metallic</t>
+  </si>
+  <si>
+    <t>Droste</t>
+  </si>
+  <si>
+    <t>Raytracing</t>
+  </si>
+  <si>
+    <t>Mandelbulb</t>
+  </si>
+  <si>
     <t>Field as string</t>
   </si>
   <si>
@@ -731,7 +768,16 @@
     <t>Decl as plain object</t>
   </si>
   <si>
-    <t>Ignore typed without valueOf()</t>
+    <t>Return value as string</t>
+  </si>
+  <si>
+    <t>Return value as typed array</t>
+  </si>
+  <si>
+    <t>Return value as clamped array</t>
+  </si>
+  <si>
+    <t>Return value as plain object</t>
   </si>
   <si>
     <t>Omitting functions</t>
@@ -806,7 +852,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -821,7 +867,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -836,7 +882,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -852,7 +898,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779145613" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -874,7 +920,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -885,7 +931,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -896,7 +942,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -907,7 +953,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -918,7 +964,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -929,7 +975,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -940,7 +986,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5C5CFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -951,7 +1008,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -962,18 +1019,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5C5CFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -995,7 +1041,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
         </ext>
       </extLst>
     </border>
@@ -1014,7 +1060,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613">
+          <pm:border xmlns:pm="smNativeData" id="1779342094">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1036,7 +1082,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613">
+          <pm:border xmlns:pm="smNativeData" id="1779342094">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1060,7 +1106,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613">
+          <pm:border xmlns:pm="smNativeData" id="1779342094">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1084,7 +1130,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613">
+          <pm:border xmlns:pm="smNativeData" id="1779342094">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1108,7 +1154,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
         </ext>
       </extLst>
     </border>
@@ -1127,7 +1173,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
         </ext>
       </extLst>
     </border>
@@ -1146,7 +1192,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
         </ext>
       </extLst>
     </border>
@@ -1165,7 +1211,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
         </ext>
       </extLst>
     </border>
@@ -1184,7 +1230,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
         </ext>
       </extLst>
     </border>
@@ -1203,7 +1249,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779145613"/>
+          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
         </ext>
       </extLst>
     </border>
@@ -1216,7 +1262,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1253,10 +1299,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1271,13 +1314,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="42">
+  <dxfs count="47">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1290,7 +1333,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1301,7 +1344,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1314,7 +1357,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1325,7 +1368,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1338,7 +1381,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1349,7 +1392,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1362,7 +1405,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1373,7 +1416,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1386,7 +1429,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1397,7 +1440,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1410,7 +1453,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1421,7 +1464,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1434,7 +1477,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1445,7 +1488,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1458,7 +1501,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1469,7 +1512,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1482,7 +1525,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1493,7 +1536,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1506,7 +1549,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1517,7 +1560,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1530,7 +1573,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1541,7 +1584,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1554,7 +1597,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1565,7 +1608,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1578,7 +1621,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1589,7 +1632,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1602,7 +1645,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1613,7 +1656,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1626,7 +1669,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1637,7 +1680,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1650,7 +1693,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1661,7 +1704,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1674,7 +1717,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1685,7 +1728,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1698,7 +1741,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1709,7 +1752,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1722,7 +1765,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1733,7 +1776,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1746,7 +1789,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1757,7 +1800,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1770,7 +1813,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1781,7 +1824,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1794,7 +1837,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1805,7 +1848,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1818,7 +1861,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1829,7 +1872,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1842,7 +1885,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1853,7 +1896,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1866,7 +1909,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1877,7 +1920,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1890,7 +1933,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1901,7 +1944,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1914,7 +1957,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1925,7 +1968,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1938,7 +1981,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1949,7 +1992,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1962,7 +2005,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1973,7 +2016,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1986,7 +2029,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1997,7 +2040,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2010,7 +2053,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2021,7 +2064,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2034,7 +2077,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2045,7 +2088,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2058,7 +2101,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2069,7 +2112,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2082,7 +2125,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2093,7 +2136,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2106,7 +2149,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2117,7 +2160,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2130,7 +2173,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2141,7 +2184,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2154,7 +2197,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2165,7 +2208,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2178,7 +2221,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2189,7 +2232,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2202,7 +2245,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2213,7 +2256,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2226,7 +2269,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2237,7 +2280,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2250,7 +2293,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2261,7 +2304,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779145613" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2274,7 +2317,127 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779145613" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2284,10 +2447,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1779145613" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1779342094" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1779145613" count="8">
+      <pm:colors xmlns:pm="smNativeData" id="1779342094" count="8">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3718,7 +3881,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3727,14 +3890,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3824,7 +3987,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3835,14 +3998,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3853,11 +4016,11 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D114"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="68.473214" customWidth="1" style="0"/>
-    <col min="4" max="4" width="12.419643" customWidth="1" style="18"/>
+    <col min="4" max="4" width="12.419643" customWidth="1" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -4153,14 +4316,13 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:2">
       <c r="A38" s="9" t="s">
         <v>146</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D38" s="13"/>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
@@ -4411,7 +4573,7 @@
       <c r="A70" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="B70" s="17"/>
+      <c r="B70" s="16"/>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="9" t="s">
@@ -4500,19 +4662,16 @@
       <c r="B81" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D81" s="18" t="s">
+      <c r="D81" s="13" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:2">
       <c r="A82" s="9" t="s">
         <v>190</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="D82" s="16" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -4522,16 +4681,19 @@
       <c r="B83" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D83" s="16" t="s">
+      <c r="D83" s="13" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
+    <row r="84" spans="1:4">
       <c r="A84" s="9" t="s">
         <v>192</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>26</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -4550,14 +4712,13 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:2">
       <c r="A87" s="9" t="s">
         <v>195</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D87" s="16"/>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="9" t="s">
@@ -4579,55 +4740,59 @@
       <c r="A90" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="B90" s="15"/>
+      <c r="B90" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="B91" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B91" s="15"/>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B92" s="15"/>
+      <c r="B92" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="B93" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B93" s="15"/>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="B94" s="15"/>
+      <c r="B94" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="B95" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B95" s="15"/>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="B96" s="10"/>
+      <c r="B96" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="B97" s="10"/>
+      <c r="B97" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="9" t="s">
@@ -4677,57 +4842,54 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:4">
+    <row r="104" spans="1:2">
       <c r="A104" s="9" t="s">
         <v>212</v>
       </c>
       <c r="B104" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D104" s="16"/>
-    </row>
-    <row r="105" spans="1:4">
+    </row>
+    <row r="105" spans="1:2">
       <c r="A105" s="9" t="s">
         <v>213</v>
       </c>
       <c r="B105" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D105" s="16"/>
-    </row>
-    <row r="106" spans="1:4">
+    </row>
+    <row r="106" spans="1:2">
       <c r="A106" s="9" t="s">
         <v>214</v>
       </c>
       <c r="B106" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D106" s="16"/>
-    </row>
-    <row r="107" spans="1:4">
+    </row>
+    <row r="107" spans="1:2">
       <c r="A107" s="9" t="s">
         <v>215</v>
       </c>
       <c r="B107" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D107" s="16" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2">
+    </row>
+    <row r="108" spans="1:4">
       <c r="A108" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="B108" s="15"/>
+      <c r="B108" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D108" s="13" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B109" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B109" s="15"/>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="9" t="s">
@@ -4766,6 +4928,38 @@
         <v>222</v>
       </c>
       <c r="B114" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="B115" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="B116" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="B117" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="B118" s="10" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4774,45 +4968,50 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B74:B114">
+  <conditionalFormatting sqref="B116:B118">
     <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43:B73">
+  <conditionalFormatting sqref="B74:B115">
     <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43:B73">
     <cfRule type="cellIs" dxfId="37" priority="3" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:B73">
+    <cfRule type="cellIs" dxfId="38" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B42">
-    <cfRule type="cellIs" dxfId="38" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="5" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B42">
-    <cfRule type="cellIs" dxfId="39" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="6" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B26">
-    <cfRule type="cellIs" dxfId="40" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="7" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B26">
-    <cfRule type="cellIs" dxfId="41" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="8" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4823,14 +5022,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4841,85 +5040,121 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B1" s="12"/>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="D1" s="17"/>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="6"/>
       <c r="B2" s="12"/>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="D2" s="17"/>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="B3" s="10"/>
-    </row>
-    <row r="4" spans="1:2">
+        <v>227</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="17"/>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="B4" s="10"/>
-    </row>
-    <row r="5" spans="1:2">
+        <v>228</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="17"/>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="B5" s="10"/>
-    </row>
-    <row r="6" spans="1:2">
+        <v>229</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="17"/>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="B6" s="10"/>
-    </row>
-    <row r="7" spans="1:2">
+        <v>230</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="17"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="B7" s="10"/>
-    </row>
-    <row r="8" spans="1:2">
+        <v>231</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="17"/>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="B8" s="10"/>
-    </row>
-    <row r="9" spans="1:2">
+        <v>232</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="B9" s="10"/>
-    </row>
-    <row r="10" spans="1:2">
+        <v>233</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="B10" s="10"/>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="B11" s="10"/>
+        <v>234</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>92</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B10">
+    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B10">
+    <cfRule type="cellIs" dxfId="44" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4930,14 +5165,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4948,7 +5183,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
@@ -4966,31 +5201,119 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="B3" s="10"/>
+        <v>235</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="B4" s="10"/>
+        <v>236</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="B5" s="10"/>
+        <v>237</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B14">
+    <cfRule type="cellIs" dxfId="45" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B14">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5001,14 +5324,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5018,6 +5341,83 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15.40"/>
+  <cols>
+    <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="12"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="6"/>
+      <c r="B2" s="12"/>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+  </mergeCells>
+  <printOptions>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+      </ext>
+    </extLst>
+  </printOptions>
+  <pageMargins left="0.787500" right="0.787500" top="1.052778" bottom="1.052778" header="0.787500" footer="0.787500"/>
+  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" cellComments="asDisplayed"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+      </ext>
+    </extLst>
+  </headerFooter>
+  <extLst>
+    <ext uri="smNativeData">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+        <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+        <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+      </pm:sheetPrefs>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="9" defaultColWidth="10.000000" defaultRowHeight="15.40"/>
@@ -5038,7 +5438,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5046,7 +5446,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5054,7 +5454,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5062,7 +5462,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5070,7 +5470,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5078,7 +5478,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5086,7 +5486,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5094,7 +5494,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5102,7 +5502,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -5110,7 +5510,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -5118,7 +5518,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -5126,7 +5526,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -5140,7 +5540,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5149,14 +5549,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5240,7 +5640,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5251,14 +5651,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5349,7 +5749,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5360,14 +5760,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5406,7 +5806,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5417,14 +5817,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5763,7 +6163,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5774,14 +6174,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5852,7 +6252,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5863,14 +6263,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5951,7 +6351,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5962,14 +6362,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6081,7 +6481,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6092,14 +6492,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6110,10 +6510,11 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
+    <col min="4" max="4" width="8.669643" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6130,13 +6531,20 @@
       <c r="A3" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="10"/>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
@@ -6174,7 +6582,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779145613" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6185,14 +6593,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779145613" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779145613" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Implemented auto release of callback functions (#968)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="11" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
+    <workbookView activeTab="5" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -27,17 +27,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1779342094" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1779342094" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1779342094" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1779342094"/>
+      <pm:revision xmlns:pm="smNativeData" day="1781256065" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1781256065" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1781256065" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1781256065"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="277">
   <si>
     <t>Context</t>
   </si>
@@ -291,6 +291,9 @@
     <t>Free function thunk</t>
   </si>
   <si>
+    <t>Free function thunk automatically at end of request</t>
+  </si>
+  <si>
     <t>Floatng point args</t>
   </si>
   <si>
@@ -303,6 +306,33 @@
     <t>Slice args</t>
   </si>
   <si>
+    <t>String args</t>
+  </si>
+  <si>
+    <t>Pass allocator as argument and return a new slice</t>
+  </si>
+  <si>
+    <t>Pass abort signal as argument</t>
+  </si>
+  <si>
+    <t>Pass promise as argument</t>
+  </si>
+  <si>
+    <t>Pass allocator and promiseas arguments</t>
+  </si>
+  <si>
+    <t>Pass generator as argument</t>
+  </si>
+  <si>
+    <t>Pass generator with allocator as argument</t>
+  </si>
+  <si>
+    <t>Throw when PHP function is used as target of pointer to variadic function</t>
+  </si>
+  <si>
+    <t>Receive transformed arguments through callback</t>
+  </si>
+  <si>
     <t>Create internal slice</t>
   </si>
   <si>
@@ -718,6 +748,21 @@
   </si>
   <si>
     <t>Get terminal name using libc function</t>
+  </si>
+  <si>
+    <t>Truncate file using posix function</t>
+  </si>
+  <si>
+    <t>Truncate opened file using posix function</t>
+  </si>
+  <si>
+    <t>Truncate opened file using win32 function</t>
+  </si>
+  <si>
+    <t>Copy real file to virtual file using copy_file_range</t>
+  </si>
+  <si>
+    <t>Copy virtual file to real file file using copy_file_range</t>
   </si>
   <si>
     <t>Basic rendering</t>
@@ -852,7 +897,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -867,7 +912,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -882,7 +927,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -898,7 +943,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779342094" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -907,7 +952,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -920,7 +965,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -931,7 +976,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -942,7 +987,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -953,7 +998,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -964,7 +1009,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -975,7 +1020,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -986,7 +1031,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -997,7 +1042,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1008,7 +1053,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1019,13 +1075,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -1041,7 +1097,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
         </ext>
       </extLst>
     </border>
@@ -1060,7 +1116,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094">
+          <pm:border xmlns:pm="smNativeData" id="1781256065">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1082,7 +1138,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094">
+          <pm:border xmlns:pm="smNativeData" id="1781256065">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1106,7 +1162,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094">
+          <pm:border xmlns:pm="smNativeData" id="1781256065">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1130,7 +1186,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094">
+          <pm:border xmlns:pm="smNativeData" id="1781256065">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1154,7 +1210,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
         </ext>
       </extLst>
     </border>
@@ -1173,7 +1229,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
         </ext>
       </extLst>
     </border>
@@ -1192,7 +1248,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
         </ext>
       </extLst>
     </border>
@@ -1211,7 +1267,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
         </ext>
       </extLst>
     </border>
@@ -1230,7 +1286,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
         </ext>
       </extLst>
     </border>
@@ -1249,7 +1305,26 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779342094"/>
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
         </ext>
       </extLst>
     </border>
@@ -1314,13 +1389,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="47">
+  <dxfs count="51">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1333,7 +1408,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1344,7 +1419,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1357,7 +1432,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1368,7 +1443,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1381,7 +1456,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1392,7 +1467,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1405,7 +1480,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1416,7 +1491,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1429,7 +1504,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1440,7 +1515,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1453,7 +1528,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1464,7 +1539,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1477,7 +1552,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1488,7 +1563,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1501,7 +1576,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1512,7 +1587,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1525,7 +1600,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1536,7 +1611,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1549,7 +1624,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1560,7 +1635,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1573,7 +1648,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1584,7 +1659,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1597,7 +1672,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1608,7 +1683,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1621,7 +1696,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1632,7 +1707,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1645,7 +1720,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1656,7 +1731,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1669,7 +1744,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1680,7 +1755,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1693,7 +1768,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1704,7 +1779,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1717,7 +1792,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1728,7 +1803,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1741,7 +1816,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1752,7 +1827,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1765,7 +1840,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1776,7 +1851,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1789,7 +1864,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1800,7 +1875,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1813,7 +1888,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1824,7 +1899,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1837,7 +1912,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1848,7 +1923,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1861,7 +1936,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1872,7 +1947,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1885,7 +1960,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1896,7 +1971,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1909,7 +1984,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1920,7 +1995,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1933,7 +2008,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1944,7 +2019,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1957,7 +2032,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1968,7 +2043,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1981,7 +2056,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1992,7 +2067,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2005,7 +2080,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2016,7 +2091,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2029,7 +2104,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2040,7 +2115,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2053,7 +2128,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2064,7 +2139,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2077,7 +2152,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2088,7 +2163,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2101,7 +2176,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2112,7 +2187,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2125,7 +2200,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2136,7 +2211,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2149,7 +2224,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2160,7 +2235,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2173,7 +2248,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2184,7 +2259,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2197,7 +2272,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2208,7 +2283,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2221,7 +2296,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2232,7 +2307,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2245,7 +2320,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2256,7 +2331,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2269,7 +2344,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2280,7 +2355,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2293,7 +2368,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2304,7 +2379,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2317,7 +2392,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2328,7 +2403,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2341,7 +2416,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2352,7 +2427,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2365,7 +2440,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2376,7 +2451,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2389,7 +2464,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2400,7 +2475,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2413,7 +2488,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2424,7 +2499,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1779342094" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2437,7 +2512,103 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1779342094" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2447,10 +2618,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1779342094" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1781256065" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1779342094" count="8">
+      <pm:colors xmlns:pm="smNativeData" id="1781256065" count="8">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -3881,7 +4052,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3890,14 +4061,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3926,7 +4097,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3935,7 +4106,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3944,7 +4115,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3953,7 +4124,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -3962,7 +4133,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -3975,19 +4146,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="33" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3998,14 +4169,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4016,7 +4187,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D118"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="68.473214" customWidth="1" style="0"/>
@@ -4035,7 +4206,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4043,7 +4214,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4051,7 +4222,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4059,7 +4230,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -4067,7 +4238,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4075,7 +4246,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -4083,7 +4254,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -4091,7 +4262,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -4099,7 +4270,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -4107,7 +4278,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -4115,18 +4286,18 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="9" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -4134,7 +4305,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>26</v>
@@ -4142,19 +4313,19 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="B16" s="15"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B17" s="15"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>26</v>
@@ -4162,7 +4333,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>26</v>
@@ -4170,7 +4341,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>26</v>
@@ -4178,18 +4349,18 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
@@ -4197,7 +4368,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
@@ -4205,7 +4376,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="9" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>26</v>
@@ -4213,7 +4384,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="9" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>26</v>
@@ -4221,13 +4392,13 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="9" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B26" s="15"/>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="9" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>28</v>
@@ -4235,7 +4406,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="9" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>26</v>
@@ -4243,7 +4414,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="9" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>26</v>
@@ -4251,7 +4422,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>26</v>
@@ -4259,7 +4430,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="9" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>26</v>
@@ -4267,7 +4438,7 @@
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="9" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>26</v>
@@ -4275,7 +4446,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="9" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>26</v>
@@ -4283,7 +4454,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="9" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>26</v>
@@ -4291,7 +4462,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="9" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>26</v>
@@ -4299,7 +4470,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="9" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>26</v>
@@ -4307,18 +4478,18 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="9" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="9" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>26</v>
@@ -4326,7 +4497,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>26</v>
@@ -4334,7 +4505,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="9" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>26</v>
@@ -4342,7 +4513,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="9" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>26</v>
@@ -4350,19 +4521,19 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="9" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B42" s="15"/>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="9" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="B43" s="15"/>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="9" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>26</v>
@@ -4370,13 +4541,13 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="9" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="B45" s="15"/>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="9" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>26</v>
@@ -4384,7 +4555,7 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="9" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>26</v>
@@ -4392,7 +4563,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="9" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>26</v>
@@ -4400,7 +4571,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="9" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>26</v>
@@ -4408,18 +4579,18 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="9" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="9" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>26</v>
@@ -4427,7 +4598,7 @@
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="9" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>26</v>
@@ -4435,7 +4606,7 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="9" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>26</v>
@@ -4443,7 +4614,7 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="9" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>26</v>
@@ -4451,7 +4622,7 @@
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="9" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>26</v>
@@ -4459,7 +4630,7 @@
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="9" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>26</v>
@@ -4467,7 +4638,7 @@
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="9" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>26</v>
@@ -4475,7 +4646,7 @@
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="9" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>26</v>
@@ -4483,7 +4654,7 @@
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="9" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>26</v>
@@ -4491,7 +4662,7 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="9" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>26</v>
@@ -4499,7 +4670,7 @@
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="9" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>26</v>
@@ -4507,7 +4678,7 @@
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="9" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>26</v>
@@ -4515,7 +4686,7 @@
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="9" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>26</v>
@@ -4523,7 +4694,7 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="9" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>26</v>
@@ -4531,7 +4702,7 @@
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="9" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>26</v>
@@ -4539,7 +4710,7 @@
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="9" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>26</v>
@@ -4547,7 +4718,7 @@
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="9" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>26</v>
@@ -4555,7 +4726,7 @@
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="9" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>26</v>
@@ -4563,7 +4734,7 @@
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="9" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>26</v>
@@ -4571,13 +4742,13 @@
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="9" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="B70" s="16"/>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="9" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>26</v>
@@ -4585,7 +4756,7 @@
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="9" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>26</v>
@@ -4593,7 +4764,7 @@
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="9" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="B73" s="10" t="s">
         <v>26</v>
@@ -4601,7 +4772,7 @@
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="9" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="B74" s="10" t="s">
         <v>26</v>
@@ -4609,7 +4780,7 @@
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="9" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>26</v>
@@ -4617,7 +4788,7 @@
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="9" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>26</v>
@@ -4625,7 +4796,7 @@
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="9" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>26</v>
@@ -4633,7 +4804,7 @@
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="9" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="B78" s="10" t="s">
         <v>26</v>
@@ -4641,7 +4812,7 @@
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="9" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="B79" s="10" t="s">
         <v>26</v>
@@ -4649,7 +4820,7 @@
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="9" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>26</v>
@@ -4657,18 +4828,18 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="9" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="9" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>26</v>
@@ -4676,29 +4847,29 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="9" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="9" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>26</v>
@@ -4706,7 +4877,7 @@
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="9" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>26</v>
@@ -4714,7 +4885,7 @@
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="9" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>26</v>
@@ -4722,7 +4893,7 @@
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="9" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>26</v>
@@ -4730,7 +4901,7 @@
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="9" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>26</v>
@@ -4738,7 +4909,7 @@
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="9" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="B90" s="10" t="s">
         <v>26</v>
@@ -4746,13 +4917,13 @@
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="B91" s="15"/>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="9" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="B92" s="10" t="s">
         <v>26</v>
@@ -4760,13 +4931,13 @@
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="B93" s="15"/>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="9" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="B94" s="10" t="s">
         <v>26</v>
@@ -4774,13 +4945,13 @@
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="B95" s="15"/>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="9" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="B96" s="10" t="s">
         <v>26</v>
@@ -4788,7 +4959,7 @@
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="9" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="B97" s="10" t="s">
         <v>26</v>
@@ -4796,7 +4967,7 @@
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="9" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="B98" s="10" t="s">
         <v>26</v>
@@ -4804,7 +4975,7 @@
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="9" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="B99" s="10" t="s">
         <v>26</v>
@@ -4812,7 +4983,7 @@
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="9" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="B100" s="10" t="s">
         <v>26</v>
@@ -4820,7 +4991,7 @@
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="9" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="B101" s="10" t="s">
         <v>26</v>
@@ -4828,7 +4999,7 @@
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="9" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="B102" s="10" t="s">
         <v>26</v>
@@ -4836,7 +5007,7 @@
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="9" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="B103" s="10" t="s">
         <v>26</v>
@@ -4844,7 +5015,7 @@
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="9" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B104" s="10" t="s">
         <v>26</v>
@@ -4852,7 +5023,7 @@
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="9" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="B105" s="10" t="s">
         <v>26</v>
@@ -4860,7 +5031,7 @@
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="9" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B106" s="10" t="s">
         <v>26</v>
@@ -4868,7 +5039,7 @@
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="9" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="B107" s="10" t="s">
         <v>26</v>
@@ -4876,24 +5047,24 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="9" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B108" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="B109" s="15"/>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="9" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="B110" s="10" t="s">
         <v>26</v>
@@ -4901,7 +5072,7 @@
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="9" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="B111" s="10" t="s">
         <v>26</v>
@@ -4909,7 +5080,7 @@
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="9" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="B112" s="10" t="s">
         <v>26</v>
@@ -4917,7 +5088,7 @@
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="9" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="B113" s="10" t="s">
         <v>26</v>
@@ -4925,7 +5096,7 @@
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="9" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B114" s="10" t="s">
         <v>26</v>
@@ -4933,7 +5104,7 @@
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="9" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="B115" s="10" t="s">
         <v>26</v>
@@ -4941,7 +5112,7 @@
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="9" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="B116" s="10" t="s">
         <v>26</v>
@@ -4949,7 +5120,7 @@
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="9" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="B117" s="10" t="s">
         <v>26</v>
@@ -4957,9 +5128,47 @@
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="9" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B118" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="B119" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B120" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="B121" s="16"/>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B122" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B123" s="10" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4968,50 +5177,50 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B116:B118">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
+  <conditionalFormatting sqref="B116:B123">
+    <cfRule type="cellIs" dxfId="39" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B74:B115">
-    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43:B73">
-    <cfRule type="cellIs" dxfId="37" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43:B73">
-    <cfRule type="cellIs" dxfId="38" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B42">
-    <cfRule type="cellIs" dxfId="39" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="5" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B42">
-    <cfRule type="cellIs" dxfId="40" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="6" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B26">
-    <cfRule type="cellIs" dxfId="41" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="7" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B26">
-    <cfRule type="cellIs" dxfId="42" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="8" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5022,14 +5231,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5051,89 +5260,89 @@
         <v>41</v>
       </c>
       <c r="B1" s="12"/>
-      <c r="D1" s="17"/>
+      <c r="D1" s="13"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="6"/>
       <c r="B2" s="12"/>
-      <c r="D2" s="17"/>
+      <c r="D2" s="13"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="17"/>
+      <c r="D3" s="13"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="17"/>
+      <c r="D4" s="13"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="17"/>
+      <c r="D5" s="13"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="17"/>
+      <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="17"/>
+      <c r="D7" s="13"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="17" t="s">
-        <v>92</v>
+      <c r="D8" s="13" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="9" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="17" t="s">
-        <v>92</v>
+      <c r="D9" s="13" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="9" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="17" t="s">
-        <v>92</v>
+      <c r="D10" s="13" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -5142,19 +5351,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="44" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5165,14 +5374,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5201,7 +5410,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5209,7 +5418,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5217,7 +5426,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5225,7 +5434,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5233,7 +5442,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5241,7 +5450,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5249,7 +5458,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5257,7 +5466,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5265,7 +5474,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -5273,7 +5482,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>28</v>
@@ -5281,7 +5490,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -5289,7 +5498,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -5301,19 +5510,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B14">
-    <cfRule type="cellIs" dxfId="45" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B14">
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5324,14 +5533,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5360,7 +5569,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5368,7 +5577,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5376,7 +5585,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5390,7 +5599,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5401,14 +5610,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5438,7 +5647,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5446,7 +5655,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>251</v>
+        <v>266</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5454,7 +5663,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5462,7 +5671,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5470,7 +5679,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5478,7 +5687,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5486,7 +5695,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5494,7 +5703,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5502,7 +5711,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -5510,7 +5719,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -5518,7 +5727,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -5526,7 +5735,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -5540,7 +5749,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5549,14 +5758,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5640,7 +5849,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5651,14 +5860,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5749,7 +5958,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5760,14 +5969,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5806,7 +6015,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5817,14 +6026,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6163,7 +6372,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6174,14 +6383,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6192,10 +6401,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
-    <col min="1" max="1" width="35.062500" customWidth="1" style="0"/>
+    <col min="1" max="1" width="61.848214" customWidth="1" style="0"/>
+    <col min="4" max="4" width="8.669643" style="17"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6212,47 +6422,157 @@
       <c r="A3" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="10"/>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="10"/>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="10"/>
+      <c r="B9" s="10"/>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B10:B18">
+    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10:B18">
+    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B9">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B9">
+    <cfRule type="cellIs" dxfId="28" priority="4" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6263,14 +6583,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6299,7 +6619,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -6307,7 +6627,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -6315,7 +6635,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="9" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -6324,13 +6644,13 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="8" spans="2:2">
       <c r="B8" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -6339,19 +6659,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B6">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B6">
-    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6362,14 +6682,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6398,7 +6718,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>28</v>
@@ -6406,13 +6726,13 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -6420,7 +6740,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>28</v>
@@ -6428,7 +6748,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -6436,20 +6756,20 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="B8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -6459,29 +6779,29 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="D8">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D8">
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="29" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="30" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6492,14 +6812,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6529,7 +6849,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -6537,30 +6857,30 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>102</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -6570,19 +6890,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779342094" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6593,14 +6913,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779342094" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779342094" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added test cases related to thread handling (#930)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -5,7 +5,7 @@
   <fileSharing readOnlyRecommended="0" userName="cleong"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="5" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
+    <workbookView activeTab="7" xWindow="240" yWindow="60" windowWidth="16380" windowHeight="8190" tabRatio="695"/>
   </bookViews>
   <sheets>
     <sheet name="Type handling" sheetId="1" r:id="rId4"/>
@@ -27,17 +27,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1781256065" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1781256065" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1781256065" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1781256065"/>
+      <pm:revision xmlns:pm="smNativeData" day="1781390401" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1781390401" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1781390401" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1781390401"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="291">
   <si>
     <t>Context</t>
   </si>
@@ -348,28 +348,70 @@
     <t>leak</t>
   </si>
   <si>
-    <t>Thread creation</t>
-  </si>
-  <si>
-    <t>Abort controller</t>
-  </si>
-  <si>
-    <t>Promise (int)</t>
-  </si>
-  <si>
-    <t>Promise (string)</t>
-  </si>
-  <si>
-    <t>Promise (plain object)</t>
-  </si>
-  <si>
-    <t>Callback</t>
-  </si>
-  <si>
-    <t>Thread pool</t>
-  </si>
-  <si>
-    <t>Memory allocation</t>
+    <t>Invoke callback</t>
+  </si>
+  <si>
+    <t>leaks</t>
+  </si>
+  <si>
+    <t>Invoke callback from thread pool</t>
+  </si>
+  <si>
+    <t>Receive promise (int)</t>
+  </si>
+  <si>
+    <t>Receive promise (string)</t>
+  </si>
+  <si>
+    <t>Receive promise (plain object)</t>
+  </si>
+  <si>
+    <t>Receive strings from generator</t>
+  </si>
+  <si>
+    <t>Receive strings from allocating generator</t>
+  </si>
+  <si>
+    <t>Receive plain objects from generator</t>
+  </si>
+  <si>
+    <t>Immediately provide value</t>
+  </si>
+  <si>
+    <t>Reject promise synchronously</t>
+  </si>
+  <si>
+    <t>Accept abort signal</t>
+  </si>
+  <si>
+    <t>Accept abort signal that works atomically</t>
+  </si>
+  <si>
+    <t>Allocate memory</t>
+  </si>
+  <si>
+    <t>Returning promise from thread pool</t>
+  </si>
+  <si>
+    <t>Call functions through work queue</t>
+  </si>
+  <si>
+    <t>Call functions through single-thread work queue</t>
+  </si>
+  <si>
+    <t>Invoke thread start function</t>
+  </si>
+  <si>
+    <t>Initialize work queue automatically</t>
+  </si>
+  <si>
+    <t>Fail to compile function with abort signal without promise</t>
+  </si>
+  <si>
+    <t>Create detached thread using pthread</t>
+  </si>
+  <si>
+    <t>Create thread within a thread using pthread</t>
   </si>
   <si>
     <t>Using ziglua</t>
@@ -897,7 +939,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -912,7 +954,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -927,7 +969,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -943,7 +985,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781256065" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -965,7 +1007,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -976,7 +1018,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -987,7 +1029,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -998,7 +1040,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1009,7 +1051,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1020,7 +1062,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1031,7 +1073,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1042,7 +1084,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1053,7 +1095,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1064,7 +1106,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1075,7 +1117,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1097,7 +1139,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1116,7 +1158,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065">
+          <pm:border xmlns:pm="smNativeData" id="1781390401">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1138,7 +1180,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065">
+          <pm:border xmlns:pm="smNativeData" id="1781390401">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1162,7 +1204,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065">
+          <pm:border xmlns:pm="smNativeData" id="1781390401">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1186,7 +1228,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065">
+          <pm:border xmlns:pm="smNativeData" id="1781390401">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1210,7 +1252,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1229,7 +1271,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1248,7 +1290,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1267,7 +1309,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1286,7 +1328,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1305,7 +1347,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1324,7 +1366,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781256065"/>
+          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
         </ext>
       </extLst>
     </border>
@@ -1337,7 +1379,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1380,6 +1422,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -1389,13 +1434,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="51">
+  <dxfs count="53">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1408,7 +1453,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1419,7 +1464,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1432,7 +1477,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1443,7 +1488,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1456,7 +1501,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1467,7 +1512,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1480,7 +1525,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1491,7 +1536,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1504,7 +1549,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1515,7 +1560,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1528,7 +1573,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1539,7 +1584,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1552,7 +1597,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1563,7 +1608,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1576,7 +1621,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1587,7 +1632,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1600,7 +1645,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1611,7 +1656,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1624,7 +1669,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1635,7 +1680,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1648,7 +1693,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1659,7 +1704,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1672,7 +1717,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1683,7 +1728,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1696,7 +1741,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1707,7 +1752,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1720,7 +1765,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1731,7 +1776,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1744,7 +1789,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1755,7 +1800,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1768,7 +1813,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1779,7 +1824,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1792,7 +1837,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1803,7 +1848,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1816,7 +1861,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1827,7 +1872,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1840,7 +1885,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1851,7 +1896,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1864,7 +1909,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1875,7 +1920,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1888,7 +1933,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1899,7 +1944,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1912,7 +1957,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1923,7 +1968,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1936,7 +1981,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1947,7 +1992,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1960,7 +2005,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1971,7 +2016,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1984,7 +2029,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1995,7 +2040,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2008,7 +2053,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2019,7 +2064,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2032,7 +2077,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2043,7 +2088,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2056,7 +2101,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2067,7 +2112,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2080,7 +2125,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2091,7 +2136,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2104,7 +2149,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2115,7 +2160,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2128,7 +2173,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2139,7 +2184,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2152,7 +2197,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2163,7 +2208,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2176,7 +2221,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2187,7 +2232,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2200,7 +2245,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2211,7 +2256,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2224,7 +2269,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2235,7 +2280,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2248,7 +2293,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2259,7 +2304,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2272,7 +2317,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2283,7 +2328,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2296,7 +2341,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2307,7 +2352,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2320,7 +2365,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2331,7 +2376,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2344,7 +2389,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2355,7 +2400,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2368,7 +2413,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2379,7 +2424,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2392,7 +2437,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2403,7 +2448,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2416,7 +2461,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2427,7 +2472,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2440,7 +2485,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2451,7 +2496,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2464,7 +2509,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2475,7 +2520,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2488,7 +2533,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2499,7 +2544,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2512,7 +2557,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2523,7 +2568,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2536,7 +2581,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2547,7 +2592,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2560,7 +2605,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2571,7 +2616,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2584,7 +2629,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2595,7 +2640,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781256065" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2608,7 +2653,55 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781256065" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2618,10 +2711,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1781256065" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1781390401" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1781256065" count="8">
+      <pm:colors xmlns:pm="smNativeData" id="1781390401" count="8">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -4052,7 +4145,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4061,14 +4154,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4097,7 +4190,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4106,7 +4199,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4115,7 +4208,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4124,7 +4217,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -4133,7 +4226,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4146,19 +4239,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="37" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="38" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4169,14 +4262,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4206,7 +4299,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4214,7 +4307,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4222,7 +4315,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4230,7 +4323,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -4238,7 +4331,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4246,7 +4339,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -4254,7 +4347,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -4262,7 +4355,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -4270,7 +4363,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -4278,7 +4371,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -4286,7 +4379,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="9" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -4297,7 +4390,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -4305,7 +4398,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>26</v>
@@ -4313,19 +4406,19 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="B16" s="15"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B17" s="15"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>26</v>
@@ -4333,7 +4426,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>26</v>
@@ -4341,7 +4434,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>26</v>
@@ -4349,7 +4442,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>26</v>
@@ -4360,7 +4453,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
@@ -4368,7 +4461,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
@@ -4376,7 +4469,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="9" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>26</v>
@@ -4384,7 +4477,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="9" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>26</v>
@@ -4392,13 +4485,13 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="9" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="B26" s="15"/>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="9" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>28</v>
@@ -4406,7 +4499,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="9" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>26</v>
@@ -4414,7 +4507,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="9" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>26</v>
@@ -4422,7 +4515,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>26</v>
@@ -4430,7 +4523,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="9" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>26</v>
@@ -4438,7 +4531,7 @@
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="9" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>26</v>
@@ -4446,7 +4539,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="9" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>26</v>
@@ -4454,7 +4547,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="9" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>26</v>
@@ -4462,7 +4555,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="9" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>26</v>
@@ -4470,7 +4563,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="9" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>26</v>
@@ -4478,7 +4571,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="9" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>26</v>
@@ -4489,7 +4582,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="9" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>26</v>
@@ -4497,7 +4590,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>26</v>
@@ -4505,7 +4598,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="9" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>26</v>
@@ -4513,7 +4606,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="9" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>26</v>
@@ -4521,19 +4614,19 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="9" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="B42" s="15"/>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="9" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="B43" s="15"/>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="9" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>26</v>
@@ -4541,13 +4634,13 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="9" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="B45" s="15"/>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="9" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>26</v>
@@ -4555,7 +4648,7 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="9" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>26</v>
@@ -4563,7 +4656,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="9" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>26</v>
@@ -4571,7 +4664,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="9" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>26</v>
@@ -4579,7 +4672,7 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="9" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>26</v>
@@ -4590,7 +4683,7 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="9" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>26</v>
@@ -4598,7 +4691,7 @@
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="9" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>26</v>
@@ -4606,7 +4699,7 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="9" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>26</v>
@@ -4614,7 +4707,7 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="9" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>26</v>
@@ -4622,7 +4715,7 @@
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="9" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>26</v>
@@ -4630,7 +4723,7 @@
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="9" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>26</v>
@@ -4638,7 +4731,7 @@
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="9" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>26</v>
@@ -4646,7 +4739,7 @@
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="9" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>26</v>
@@ -4654,7 +4747,7 @@
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="9" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>26</v>
@@ -4662,7 +4755,7 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="9" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>26</v>
@@ -4670,7 +4763,7 @@
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="9" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>26</v>
@@ -4678,7 +4771,7 @@
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="9" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>26</v>
@@ -4686,7 +4779,7 @@
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="9" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>26</v>
@@ -4694,7 +4787,7 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="9" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>26</v>
@@ -4702,7 +4795,7 @@
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="9" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>26</v>
@@ -4710,7 +4803,7 @@
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="9" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>26</v>
@@ -4718,7 +4811,7 @@
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="9" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>26</v>
@@ -4726,7 +4819,7 @@
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="9" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>26</v>
@@ -4734,7 +4827,7 @@
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="9" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>26</v>
@@ -4742,13 +4835,13 @@
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="9" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="B70" s="16"/>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="9" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>26</v>
@@ -4756,7 +4849,7 @@
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="9" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>26</v>
@@ -4764,7 +4857,7 @@
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="9" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="B73" s="10" t="s">
         <v>26</v>
@@ -4772,7 +4865,7 @@
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="9" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="B74" s="10" t="s">
         <v>26</v>
@@ -4780,7 +4873,7 @@
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="9" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>26</v>
@@ -4788,7 +4881,7 @@
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="9" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>26</v>
@@ -4796,7 +4889,7 @@
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="9" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>26</v>
@@ -4804,7 +4897,7 @@
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="9" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="B78" s="10" t="s">
         <v>26</v>
@@ -4812,7 +4905,7 @@
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="9" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="B79" s="10" t="s">
         <v>26</v>
@@ -4820,7 +4913,7 @@
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="9" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>26</v>
@@ -4828,7 +4921,7 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="9" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>26</v>
@@ -4839,7 +4932,7 @@
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="9" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>26</v>
@@ -4847,7 +4940,7 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="9" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>26</v>
@@ -4858,7 +4951,7 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="9" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>26</v>
@@ -4869,7 +4962,7 @@
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="9" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>26</v>
@@ -4877,7 +4970,7 @@
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="9" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>26</v>
@@ -4885,7 +4978,7 @@
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="9" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>26</v>
@@ -4893,7 +4986,7 @@
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="9" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>26</v>
@@ -4901,7 +4994,7 @@
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="9" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>26</v>
@@ -4909,7 +5002,7 @@
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="9" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="B90" s="10" t="s">
         <v>26</v>
@@ -4917,13 +5010,13 @@
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B91" s="15"/>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="9" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="B92" s="10" t="s">
         <v>26</v>
@@ -4931,13 +5024,13 @@
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="B93" s="15"/>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="9" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="B94" s="10" t="s">
         <v>26</v>
@@ -4945,13 +5038,13 @@
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="B95" s="15"/>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="9" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="B96" s="10" t="s">
         <v>26</v>
@@ -4959,7 +5052,7 @@
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="9" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B97" s="10" t="s">
         <v>26</v>
@@ -4967,7 +5060,7 @@
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="9" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="B98" s="10" t="s">
         <v>26</v>
@@ -4975,7 +5068,7 @@
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="9" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="B99" s="10" t="s">
         <v>26</v>
@@ -4983,7 +5076,7 @@
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="9" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="B100" s="10" t="s">
         <v>26</v>
@@ -4991,7 +5084,7 @@
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="9" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="B101" s="10" t="s">
         <v>26</v>
@@ -4999,7 +5092,7 @@
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="9" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="B102" s="10" t="s">
         <v>26</v>
@@ -5007,7 +5100,7 @@
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="9" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="B103" s="10" t="s">
         <v>26</v>
@@ -5015,7 +5108,7 @@
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="9" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="B104" s="10" t="s">
         <v>26</v>
@@ -5023,7 +5116,7 @@
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="9" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="B105" s="10" t="s">
         <v>26</v>
@@ -5031,7 +5124,7 @@
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="9" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="B106" s="10" t="s">
         <v>26</v>
@@ -5039,7 +5132,7 @@
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="9" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="B107" s="10" t="s">
         <v>26</v>
@@ -5047,7 +5140,7 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="9" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="B108" s="10" t="s">
         <v>26</v>
@@ -5058,13 +5151,13 @@
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="B109" s="15"/>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="9" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="B110" s="10" t="s">
         <v>26</v>
@@ -5072,7 +5165,7 @@
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="9" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="B111" s="10" t="s">
         <v>26</v>
@@ -5080,7 +5173,7 @@
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="9" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="B112" s="10" t="s">
         <v>26</v>
@@ -5088,7 +5181,7 @@
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="9" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="B113" s="10" t="s">
         <v>26</v>
@@ -5096,7 +5189,7 @@
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="9" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="B114" s="10" t="s">
         <v>26</v>
@@ -5104,7 +5197,7 @@
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="9" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="B115" s="10" t="s">
         <v>26</v>
@@ -5112,7 +5205,7 @@
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="9" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="B116" s="10" t="s">
         <v>26</v>
@@ -5120,7 +5213,7 @@
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="9" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="B117" s="10" t="s">
         <v>26</v>
@@ -5128,7 +5221,7 @@
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="9" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="B118" s="10" t="s">
         <v>26</v>
@@ -5136,7 +5229,7 @@
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="9" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="B119" s="10" t="s">
         <v>26</v>
@@ -5144,7 +5237,7 @@
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="9" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="B120" s="10" t="s">
         <v>26</v>
@@ -5152,13 +5245,13 @@
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="9" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="B121" s="16"/>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="9" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="B122" s="10" t="s">
         <v>26</v>
@@ -5166,7 +5259,7 @@
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="9" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="B123" s="10" t="s">
         <v>26</v>
@@ -5178,49 +5271,49 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B116:B123">
-    <cfRule type="cellIs" dxfId="39" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B74:B115">
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="2" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43:B73">
-    <cfRule type="cellIs" dxfId="41" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43:B73">
-    <cfRule type="cellIs" dxfId="42" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B42">
-    <cfRule type="cellIs" dxfId="43" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="5" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B42">
-    <cfRule type="cellIs" dxfId="44" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="6" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B26">
-    <cfRule type="cellIs" dxfId="45" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="7" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B26">
-    <cfRule type="cellIs" dxfId="46" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="8" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5231,14 +5324,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5269,7 +5362,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5278,7 +5371,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5287,7 +5380,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5296,7 +5389,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5305,7 +5398,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5314,7 +5407,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5325,7 +5418,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="9" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5336,7 +5429,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="9" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5351,19 +5444,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B10">
-    <cfRule type="cellIs" dxfId="48" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5374,14 +5467,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5410,7 +5503,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5418,7 +5511,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5426,7 +5519,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5434,7 +5527,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5442,7 +5535,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5450,7 +5543,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5458,7 +5551,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5466,7 +5559,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5474,7 +5567,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -5482,7 +5575,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>28</v>
@@ -5490,7 +5583,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -5498,7 +5591,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -5510,19 +5603,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B14">
-    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B14">
-    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5533,14 +5626,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5569,7 +5662,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5577,7 +5670,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5585,7 +5678,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5599,7 +5692,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5610,14 +5703,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5647,7 +5740,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5655,7 +5748,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5663,7 +5756,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5671,7 +5764,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5679,7 +5772,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5687,7 +5780,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5695,7 +5788,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5703,7 +5796,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5711,7 +5804,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -5719,7 +5812,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -5727,7 +5820,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -5735,7 +5828,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -5749,7 +5842,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5758,14 +5851,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5849,7 +5942,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5860,14 +5953,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5958,7 +6051,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5969,14 +6062,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6015,7 +6108,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6026,14 +6119,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6372,7 +6465,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6383,14 +6476,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6572,7 +6665,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6583,14 +6676,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6671,7 +6764,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6682,14 +6775,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6700,10 +6793,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
-    <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
+    <col min="1" max="1" width="49.187500" customWidth="1" style="0"/>
+    <col min="4" max="4" width="8.669643" style="18"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6716,92 +6810,251 @@
       <c r="A2" s="6"/>
       <c r="B2" s="12"/>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
         <v>103</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="10"/>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B8" s="10"/>
-      <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B9" s="10"/>
+        <v>110</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="B10" s="10"/>
+        <v>111</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="9"/>
+      <c r="B24" s="10"/>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="9"/>
+      <c r="B25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="D8">
+  <conditionalFormatting sqref="B15:B25">
     <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D8">
+  <conditionalFormatting sqref="B15:B25">
     <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B10">
+  <conditionalFormatting sqref="B13:B14">
     <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B10">
+  <conditionalFormatting sqref="B13:B14">
     <cfRule type="cellIs" dxfId="34" priority="4" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B12">
+    <cfRule type="cellIs" dxfId="35" priority="5" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B12">
+    <cfRule type="cellIs" dxfId="36" priority="6" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6812,14 +7065,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6849,7 +7102,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -6857,7 +7110,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -6868,19 +7121,19 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -6890,19 +7143,19 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B7">
-    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781256065" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6913,14 +7166,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781256065" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781256065" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added test cases for thread handling (#930)
</commit_message>
<xml_diff>
--- a/php-zigar/test/test-matrix.xlsx
+++ b/php-zigar/test/test-matrix.xlsx
@@ -27,17 +27,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1781390401" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1781390401" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1781390401" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1781390401"/>
+      <pm:revision xmlns:pm="smNativeData" day="1781562667" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1781562667" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1781562667" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1781562667"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="311">
   <si>
     <t>Context</t>
   </si>
@@ -412,6 +412,66 @@
   </si>
   <si>
     <t>Create thread within a thread using pthread</t>
+  </si>
+  <si>
+    <t>Exit thread created using pthread</t>
+  </si>
+  <si>
+    <t>Exit thread created in a thread using pthread</t>
+  </si>
+  <si>
+    <t>Print ids of threads creat using pthread</t>
+  </si>
+  <si>
+    <t>Create mutex using pthread</t>
+  </si>
+  <si>
+    <t>Create error checking mutex using pthread</t>
+  </si>
+  <si>
+    <t>Create recursive mutex using pthread</t>
+  </si>
+  <si>
+    <t>Wait momentarily for mutex created using pthread</t>
+  </si>
+  <si>
+    <t>Create spinlock using pthread</t>
+  </si>
+  <si>
+    <t>Create read/write lock using pthread</t>
+  </si>
+  <si>
+    <t>Wait momentarily for read lock created using pthread</t>
+  </si>
+  <si>
+    <t>Wait momentarily for write lock created using pthread</t>
+  </si>
+  <si>
+    <t>Create semaphore using pthread</t>
+  </si>
+  <si>
+    <t>Create named semaphore using pthread</t>
+  </si>
+  <si>
+    <t>Wait momentarily for semaphore created using pthread</t>
+  </si>
+  <si>
+    <t>Get semaphore created using pthread</t>
+  </si>
+  <si>
+    <t>Create key for thread specific vakue using pthread</t>
+  </si>
+  <si>
+    <t>Exit thread not created using pthread</t>
+  </si>
+  <si>
+    <t>Call function once using pthread</t>
+  </si>
+  <si>
+    <t>Create condition using pthread</t>
+  </si>
+  <si>
+    <t>Wait momentarily for condition created using pthread</t>
   </si>
   <si>
     <t>Using ziglua</t>
@@ -939,7 +999,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781562667" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -954,7 +1014,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781562667" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -969,7 +1029,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781562667" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -985,7 +1045,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1781390401" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1781562667" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -1007,7 +1067,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1018,7 +1078,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1029,7 +1089,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1040,7 +1100,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1051,7 +1111,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1062,7 +1122,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="38" fgClr="00FFFF00" bgLvl="62" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1073,7 +1133,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1084,7 +1144,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="005C5CFF" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1095,7 +1155,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1106,7 +1166,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1117,7 +1177,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1139,7 +1199,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1158,7 +1218,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401">
+          <pm:border xmlns:pm="smNativeData" id="1781562667">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1180,7 +1240,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401">
+          <pm:border xmlns:pm="smNativeData" id="1781562667">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1204,7 +1264,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401">
+          <pm:border xmlns:pm="smNativeData" id="1781562667">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1228,7 +1288,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401">
+          <pm:border xmlns:pm="smNativeData" id="1781562667">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1252,7 +1312,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1271,7 +1331,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1290,7 +1350,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1309,7 +1369,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1328,7 +1388,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1347,7 +1407,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1366,7 +1426,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1781390401"/>
+          <pm:border xmlns:pm="smNativeData" id="1781562667"/>
         </ext>
       </extLst>
     </border>
@@ -1379,7 +1439,7 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1419,12 +1479,6 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -1440,7 +1494,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1453,7 +1507,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1464,7 +1518,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1477,7 +1531,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1488,7 +1542,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1501,7 +1555,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1512,7 +1566,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1525,7 +1579,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1536,7 +1590,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1549,7 +1603,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1560,7 +1614,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1573,7 +1627,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1584,7 +1638,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1597,7 +1651,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1608,7 +1662,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1621,7 +1675,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1632,7 +1686,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1645,7 +1699,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1656,7 +1710,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1669,7 +1723,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1680,7 +1734,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1693,7 +1747,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1704,7 +1758,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1717,7 +1771,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1728,7 +1782,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1741,7 +1795,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1752,7 +1806,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1765,7 +1819,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1776,7 +1830,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1789,7 +1843,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1800,7 +1854,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1813,7 +1867,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1824,7 +1878,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1837,7 +1891,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1848,7 +1902,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1861,7 +1915,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1872,7 +1926,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1885,7 +1939,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1896,7 +1950,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1909,7 +1963,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1920,7 +1974,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1933,7 +1987,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1944,7 +1998,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1957,7 +2011,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1968,7 +2022,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1981,7 +2035,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1992,7 +2046,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2005,7 +2059,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2016,7 +2070,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2029,7 +2083,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2040,7 +2094,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2053,7 +2107,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2064,7 +2118,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2077,7 +2131,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2088,7 +2142,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2101,7 +2155,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2112,7 +2166,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2125,7 +2179,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2136,7 +2190,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2149,7 +2203,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2160,7 +2214,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2173,7 +2227,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2184,7 +2238,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2197,7 +2251,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2208,7 +2262,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2221,7 +2275,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2232,7 +2286,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2245,7 +2299,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2256,7 +2310,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2269,7 +2323,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2280,7 +2334,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2293,7 +2347,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2304,7 +2358,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2317,7 +2371,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2328,7 +2382,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2341,7 +2395,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2352,7 +2406,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2365,7 +2419,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2376,7 +2430,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2389,7 +2443,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2400,7 +2454,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2413,7 +2467,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2424,7 +2478,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2437,7 +2491,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2448,7 +2502,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2461,7 +2515,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2472,7 +2526,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2485,7 +2539,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2496,7 +2550,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2509,7 +2563,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2520,7 +2574,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2533,7 +2587,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2544,7 +2598,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2557,7 +2611,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2568,7 +2622,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2581,7 +2635,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2592,7 +2646,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2605,7 +2659,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2616,7 +2670,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2629,7 +2683,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2640,7 +2694,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2653,7 +2707,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2664,7 +2718,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2677,7 +2731,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2688,7 +2742,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1781390401" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1781562667" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -2701,7 +2755,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1781390401" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1781562667" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -2711,10 +2765,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1781390401" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1781562667" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1781390401" count="8">
+      <pm:colors xmlns:pm="smNativeData" id="1781562667" count="8">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -4145,7 +4199,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4154,14 +4208,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4190,7 +4244,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4199,7 +4253,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>131</v>
+        <v>151</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4208,7 +4262,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4217,7 +4271,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -4226,7 +4280,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4251,7 +4305,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4262,14 +4316,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4299,7 +4353,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -4307,7 +4361,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -4315,7 +4369,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -4323,7 +4377,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -4331,7 +4385,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -4339,7 +4393,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -4347,7 +4401,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -4355,7 +4409,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -4363,7 +4417,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -4371,7 +4425,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -4379,7 +4433,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="9" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -4390,7 +4444,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -4398,7 +4452,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>26</v>
@@ -4406,19 +4460,19 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="B16" s="15"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="B17" s="15"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>26</v>
@@ -4426,7 +4480,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>26</v>
@@ -4434,7 +4488,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>26</v>
@@ -4442,7 +4496,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>26</v>
@@ -4453,7 +4507,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
@@ -4461,7 +4515,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
@@ -4469,7 +4523,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="9" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>26</v>
@@ -4477,7 +4531,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="9" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>26</v>
@@ -4485,13 +4539,13 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="9" t="s">
-        <v>158</v>
+        <v>178</v>
       </c>
       <c r="B26" s="15"/>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="9" t="s">
-        <v>159</v>
+        <v>179</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>28</v>
@@ -4499,7 +4553,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="9" t="s">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>26</v>
@@ -4507,7 +4561,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="9" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>26</v>
@@ -4515,7 +4569,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>162</v>
+        <v>182</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>26</v>
@@ -4523,7 +4577,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="9" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>26</v>
@@ -4531,7 +4585,7 @@
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="9" t="s">
-        <v>164</v>
+        <v>184</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>26</v>
@@ -4539,7 +4593,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="9" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>26</v>
@@ -4547,7 +4601,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="9" t="s">
-        <v>166</v>
+        <v>186</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>26</v>
@@ -4555,7 +4609,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="9" t="s">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>26</v>
@@ -4563,7 +4617,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="9" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>26</v>
@@ -4571,7 +4625,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="9" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>26</v>
@@ -4582,7 +4636,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="9" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>26</v>
@@ -4590,7 +4644,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>26</v>
@@ -4598,7 +4652,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="9" t="s">
-        <v>172</v>
+        <v>192</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>26</v>
@@ -4606,7 +4660,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="9" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>26</v>
@@ -4614,19 +4668,19 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="9" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="B42" s="15"/>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="9" t="s">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="B43" s="15"/>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="9" t="s">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>26</v>
@@ -4634,13 +4688,13 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="9" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="B45" s="15"/>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="9" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>26</v>
@@ -4648,7 +4702,7 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="9" t="s">
-        <v>179</v>
+        <v>199</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>26</v>
@@ -4656,7 +4710,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="9" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>26</v>
@@ -4664,7 +4718,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="9" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>26</v>
@@ -4672,7 +4726,7 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="9" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>26</v>
@@ -4683,7 +4737,7 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="9" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>26</v>
@@ -4691,7 +4745,7 @@
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="9" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>26</v>
@@ -4699,7 +4753,7 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="9" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>26</v>
@@ -4707,7 +4761,7 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="9" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>26</v>
@@ -4715,7 +4769,7 @@
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="9" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>26</v>
@@ -4723,7 +4777,7 @@
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="9" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>26</v>
@@ -4731,7 +4785,7 @@
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="9" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>26</v>
@@ -4739,7 +4793,7 @@
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="9" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>26</v>
@@ -4747,7 +4801,7 @@
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="9" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>26</v>
@@ -4755,7 +4809,7 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="9" t="s">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>26</v>
@@ -4763,7 +4817,7 @@
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="9" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>26</v>
@@ -4771,7 +4825,7 @@
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="9" t="s">
-        <v>194</v>
+        <v>214</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>26</v>
@@ -4779,7 +4833,7 @@
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="9" t="s">
-        <v>195</v>
+        <v>215</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>26</v>
@@ -4787,7 +4841,7 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="9" t="s">
-        <v>196</v>
+        <v>216</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>26</v>
@@ -4795,7 +4849,7 @@
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="9" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>26</v>
@@ -4803,7 +4857,7 @@
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="9" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>26</v>
@@ -4811,7 +4865,7 @@
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="9" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>26</v>
@@ -4819,7 +4873,7 @@
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="9" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>26</v>
@@ -4827,7 +4881,7 @@
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="9" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>26</v>
@@ -4835,13 +4889,13 @@
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="9" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="B70" s="16"/>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="9" t="s">
-        <v>203</v>
+        <v>223</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>26</v>
@@ -4849,7 +4903,7 @@
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="9" t="s">
-        <v>204</v>
+        <v>224</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>26</v>
@@ -4857,7 +4911,7 @@
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="9" t="s">
-        <v>205</v>
+        <v>225</v>
       </c>
       <c r="B73" s="10" t="s">
         <v>26</v>
@@ -4865,7 +4919,7 @@
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="9" t="s">
-        <v>206</v>
+        <v>226</v>
       </c>
       <c r="B74" s="10" t="s">
         <v>26</v>
@@ -4873,7 +4927,7 @@
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="9" t="s">
-        <v>207</v>
+        <v>227</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>26</v>
@@ -4881,7 +4935,7 @@
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="9" t="s">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>26</v>
@@ -4889,7 +4943,7 @@
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="9" t="s">
-        <v>209</v>
+        <v>229</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>26</v>
@@ -4897,7 +4951,7 @@
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="9" t="s">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="B78" s="10" t="s">
         <v>26</v>
@@ -4905,7 +4959,7 @@
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="9" t="s">
-        <v>211</v>
+        <v>231</v>
       </c>
       <c r="B79" s="10" t="s">
         <v>26</v>
@@ -4913,7 +4967,7 @@
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="9" t="s">
-        <v>212</v>
+        <v>232</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>26</v>
@@ -4921,7 +4975,7 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="9" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>26</v>
@@ -4932,7 +4986,7 @@
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="9" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>26</v>
@@ -4940,7 +4994,7 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="9" t="s">
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>26</v>
@@ -4951,7 +5005,7 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="9" t="s">
-        <v>216</v>
+        <v>236</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>26</v>
@@ -4962,7 +5016,7 @@
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="9" t="s">
-        <v>217</v>
+        <v>237</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>26</v>
@@ -4970,7 +5024,7 @@
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="9" t="s">
-        <v>218</v>
+        <v>238</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>26</v>
@@ -4978,7 +5032,7 @@
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="9" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>26</v>
@@ -4986,7 +5040,7 @@
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="9" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>26</v>
@@ -4994,7 +5048,7 @@
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="9" t="s">
-        <v>221</v>
+        <v>241</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>26</v>
@@ -5002,7 +5056,7 @@
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="9" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="B90" s="10" t="s">
         <v>26</v>
@@ -5010,13 +5064,13 @@
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
-        <v>223</v>
+        <v>243</v>
       </c>
       <c r="B91" s="15"/>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="9" t="s">
-        <v>224</v>
+        <v>244</v>
       </c>
       <c r="B92" s="10" t="s">
         <v>26</v>
@@ -5024,13 +5078,13 @@
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="B93" s="15"/>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="9" t="s">
-        <v>226</v>
+        <v>246</v>
       </c>
       <c r="B94" s="10" t="s">
         <v>26</v>
@@ -5038,13 +5092,13 @@
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
-        <v>227</v>
+        <v>247</v>
       </c>
       <c r="B95" s="15"/>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="9" t="s">
-        <v>228</v>
+        <v>248</v>
       </c>
       <c r="B96" s="10" t="s">
         <v>26</v>
@@ -5052,7 +5106,7 @@
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="9" t="s">
-        <v>229</v>
+        <v>249</v>
       </c>
       <c r="B97" s="10" t="s">
         <v>26</v>
@@ -5060,7 +5114,7 @@
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="9" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B98" s="10" t="s">
         <v>26</v>
@@ -5068,7 +5122,7 @@
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="9" t="s">
-        <v>231</v>
+        <v>251</v>
       </c>
       <c r="B99" s="10" t="s">
         <v>26</v>
@@ -5076,7 +5130,7 @@
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="9" t="s">
-        <v>232</v>
+        <v>252</v>
       </c>
       <c r="B100" s="10" t="s">
         <v>26</v>
@@ -5084,7 +5138,7 @@
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="9" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="B101" s="10" t="s">
         <v>26</v>
@@ -5092,7 +5146,7 @@
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="9" t="s">
-        <v>234</v>
+        <v>254</v>
       </c>
       <c r="B102" s="10" t="s">
         <v>26</v>
@@ -5100,7 +5154,7 @@
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="9" t="s">
-        <v>235</v>
+        <v>255</v>
       </c>
       <c r="B103" s="10" t="s">
         <v>26</v>
@@ -5108,7 +5162,7 @@
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="9" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="B104" s="10" t="s">
         <v>26</v>
@@ -5116,7 +5170,7 @@
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="9" t="s">
-        <v>237</v>
+        <v>257</v>
       </c>
       <c r="B105" s="10" t="s">
         <v>26</v>
@@ -5124,7 +5178,7 @@
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="9" t="s">
-        <v>238</v>
+        <v>258</v>
       </c>
       <c r="B106" s="10" t="s">
         <v>26</v>
@@ -5132,7 +5186,7 @@
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="9" t="s">
-        <v>239</v>
+        <v>259</v>
       </c>
       <c r="B107" s="10" t="s">
         <v>26</v>
@@ -5140,7 +5194,7 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="9" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="B108" s="10" t="s">
         <v>26</v>
@@ -5151,13 +5205,13 @@
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
-        <v>241</v>
+        <v>261</v>
       </c>
       <c r="B109" s="15"/>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="9" t="s">
-        <v>242</v>
+        <v>262</v>
       </c>
       <c r="B110" s="10" t="s">
         <v>26</v>
@@ -5165,7 +5219,7 @@
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="9" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="B111" s="10" t="s">
         <v>26</v>
@@ -5173,7 +5227,7 @@
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="9" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="B112" s="10" t="s">
         <v>26</v>
@@ -5181,7 +5235,7 @@
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="9" t="s">
-        <v>245</v>
+        <v>265</v>
       </c>
       <c r="B113" s="10" t="s">
         <v>26</v>
@@ -5189,7 +5243,7 @@
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="9" t="s">
-        <v>246</v>
+        <v>266</v>
       </c>
       <c r="B114" s="10" t="s">
         <v>26</v>
@@ -5197,7 +5251,7 @@
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="9" t="s">
-        <v>247</v>
+        <v>267</v>
       </c>
       <c r="B115" s="10" t="s">
         <v>26</v>
@@ -5205,7 +5259,7 @@
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="9" t="s">
-        <v>248</v>
+        <v>268</v>
       </c>
       <c r="B116" s="10" t="s">
         <v>26</v>
@@ -5213,7 +5267,7 @@
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="9" t="s">
-        <v>249</v>
+        <v>269</v>
       </c>
       <c r="B117" s="10" t="s">
         <v>26</v>
@@ -5221,7 +5275,7 @@
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="9" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="B118" s="10" t="s">
         <v>26</v>
@@ -5229,7 +5283,7 @@
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="9" t="s">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="B119" s="10" t="s">
         <v>26</v>
@@ -5237,7 +5291,7 @@
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="9" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="B120" s="10" t="s">
         <v>26</v>
@@ -5245,13 +5299,13 @@
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="9" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="B121" s="16"/>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="9" t="s">
-        <v>254</v>
+        <v>274</v>
       </c>
       <c r="B122" s="10" t="s">
         <v>26</v>
@@ -5259,7 +5313,7 @@
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="9" t="s">
-        <v>255</v>
+        <v>275</v>
       </c>
       <c r="B123" s="10" t="s">
         <v>26</v>
@@ -5313,7 +5367,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5324,14 +5378,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5362,7 +5416,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>256</v>
+        <v>276</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5371,7 +5425,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>257</v>
+        <v>277</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5380,7 +5434,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>258</v>
+        <v>278</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5389,7 +5443,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>259</v>
+        <v>279</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5398,7 +5452,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5407,7 +5461,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5418,7 +5472,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="9" t="s">
-        <v>262</v>
+        <v>282</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5429,7 +5483,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="9" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5456,7 +5510,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5467,14 +5521,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5503,7 +5557,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5511,7 +5565,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>265</v>
+        <v>285</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5519,7 +5573,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>266</v>
+        <v>286</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5527,7 +5581,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>267</v>
+        <v>287</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5535,7 +5589,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>268</v>
+        <v>288</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5543,7 +5597,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5551,7 +5605,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5559,7 +5613,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>271</v>
+        <v>291</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5567,7 +5621,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>272</v>
+        <v>292</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -5575,7 +5629,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>273</v>
+        <v>293</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>28</v>
@@ -5583,7 +5637,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>274</v>
+        <v>294</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -5591,7 +5645,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>275</v>
+        <v>295</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -5615,7 +5669,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5626,14 +5680,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5662,7 +5716,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>276</v>
+        <v>296</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5670,7 +5724,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>277</v>
+        <v>297</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5678,7 +5732,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>278</v>
+        <v>298</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5692,7 +5746,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5703,14 +5757,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5740,7 +5794,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>279</v>
+        <v>299</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -5748,7 +5802,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -5756,7 +5810,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>281</v>
+        <v>301</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -5764,7 +5818,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>282</v>
+        <v>302</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -5772,7 +5826,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>283</v>
+        <v>303</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -5780,7 +5834,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>284</v>
+        <v>304</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -5788,7 +5842,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>285</v>
+        <v>305</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -5796,7 +5850,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>286</v>
+        <v>306</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -5804,7 +5858,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>287</v>
+        <v>307</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -5812,7 +5866,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>288</v>
+        <v>308</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -5820,7 +5874,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>289</v>
+        <v>309</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -5828,7 +5882,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -5842,7 +5896,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5851,14 +5905,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5942,7 +5996,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5953,14 +6007,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6051,7 +6105,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6062,14 +6116,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6108,7 +6162,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6119,14 +6173,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6465,7 +6519,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6476,14 +6530,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6498,7 +6552,7 @@
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="61.848214" customWidth="1" style="0"/>
-    <col min="4" max="4" width="8.669643" style="17"/>
+    <col min="4" max="4" width="8.669643" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6665,7 +6719,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6676,14 +6730,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6764,7 +6818,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6775,14 +6829,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6793,11 +6847,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
-    <col min="1" max="1" width="49.187500" customWidth="1" style="0"/>
-    <col min="4" max="4" width="8.669643" style="18"/>
+    <col min="1" max="1" width="52.401786" customWidth="1" style="0"/>
+    <col min="4" max="4" width="8.669643" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6817,52 +6871,40 @@
       <c r="B3" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="13" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
         <v>105</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="17" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
         <v>106</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="17" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
         <v>107</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="17" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
         <v>108</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -6889,26 +6931,20 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
         <v>112</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="17" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
+    </row>
+    <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
         <v>113</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -6916,7 +6952,7 @@
         <v>114</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -6924,7 +6960,7 @@
         <v>115</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -6932,18 +6968,15 @@
         <v>116</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
         <v>117</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="D16" s="17" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -6951,7 +6984,7 @@
         <v>118</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -6959,7 +6992,7 @@
         <v>119</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -6967,7 +7000,7 @@
         <v>120</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -6975,7 +7008,7 @@
         <v>121</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -6986,47 +7019,193 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
         <v>123</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
+    </row>
+    <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
         <v>124</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>104</v>
-      </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
+      <c r="A24" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="9"/>
-      <c r="B25" s="10"/>
+      <c r="A25" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B15:B25">
+  <conditionalFormatting sqref="B15:B43">
     <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:B25">
+  <conditionalFormatting sqref="B15:B43">
     <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
@@ -7054,7 +7233,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -7065,14 +7244,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -7102,7 +7281,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -7110,7 +7289,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -7121,19 +7300,19 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -7155,7 +7334,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1781390401" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1781562667" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -7166,14 +7345,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1781390401" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1781562667" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781390401" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1781562667" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>